<commit_message>
Recette : retours d'Hervé du 22/10 et réponses (classeur)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MoqekrFvgrWkuAe5NHnE5A
</commit_message>
<xml_diff>
--- a/docs/recette/RECETTE_PR_17-37.xlsx
+++ b/docs/recette/RECETTE_PR_17-37.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Tests" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,19 +11,17 @@
     <sheet name="Légende" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tests'!$A$4:$I$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tests'!$A$4:$J$33</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Tests'!$4:$4</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
-  </numFmts>
-  <fonts count="10">
+  <numFmts count="0"/>
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,12 +37,14 @@
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="00595959"/>
+      <color rgb="FF595959"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -59,11 +58,12 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="00595959"/>
+      <color rgb="FF595959"/>
       <sz val="9"/>
     </font>
     <font>
@@ -76,8 +76,13 @@
       <i val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -86,26 +91,51 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF1F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -126,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -142,7 +172,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="14" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -167,36 +197,59 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="6">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00C6EFCE"/>
+          <fgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FFC7CE"/>
+          <fgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FFEB9C"/>
+          <fgColor rgb="FFD9D9D9"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00D9D9D9"/>
+          <fgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -562,21 +615,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:J33"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="4" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="18" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Recette VERIFLOW : PR 17 à 37 (build de la branche claude/recette, Windows 11)</t>
@@ -636,8 +689,13 @@
           <t>Commentaires</t>
         </is>
       </c>
-    </row>
-    <row r="5">
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Réponse de Claude (23/10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="25.5" customHeight="1">
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
@@ -663,14 +721,25 @@
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr"/>
-      <c r="H5" s="7" t="n"/>
-      <c r="I5" s="8" t="inlineStr"/>
-    </row>
-    <row r="6">
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>RAS</t>
+        </is>
+      </c>
+      <c r="J5" s="19" t="inlineStr"/>
+    </row>
+    <row r="6" ht="25.5" customHeight="1">
       <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
@@ -696,14 +765,25 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="7" t="n"/>
-      <c r="I6" s="8" t="inlineStr"/>
-    </row>
-    <row r="7">
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>RAS</t>
+        </is>
+      </c>
+      <c r="J6" s="19" t="inlineStr"/>
+    </row>
+    <row r="7" ht="25.5" customHeight="1">
       <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
@@ -729,14 +809,25 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="7" t="n"/>
-      <c r="I7" s="8" t="inlineStr"/>
-    </row>
-    <row r="8">
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>RAS</t>
+        </is>
+      </c>
+      <c r="J7" s="19" t="inlineStr"/>
+    </row>
+    <row r="8" ht="25.5" customHeight="1">
       <c r="A8" s="4" t="n">
         <v>4</v>
       </c>
@@ -762,14 +853,29 @@
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr"/>
-      <c r="H8" s="7" t="n"/>
-      <c r="I8" s="8" t="inlineStr"/>
-    </row>
-    <row r="9">
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>Manuel assez sommaire, il faut le développer plus pour permettre l'utilisateur d'être autonome sur le logiciel</t>
+        </is>
+      </c>
+      <c r="J8" s="20" t="inlineStr">
+        <is>
+          <t>Guide développé : 12 chapitres au lieu de 7, 610 lignes au lieu de 194 (journée de tournage, recettes TRANSCODE, problèmes fréquents, glossaire). À relire dans le nouveau build.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="25.5" customHeight="1">
       <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
@@ -795,14 +901,25 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr"/>
-      <c r="H9" s="7" t="n"/>
-      <c r="I9" s="8" t="inlineStr"/>
-    </row>
-    <row r="10">
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>RAS</t>
+        </is>
+      </c>
+      <c r="J9" s="19" t="inlineStr"/>
+    </row>
+    <row r="10" ht="63.75" customHeight="1">
       <c r="A10" s="4" t="n">
         <v>6</v>
       </c>
@@ -828,12 +945,27 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr"/>
-      <c r="H10" s="7" t="n"/>
-      <c r="I10" s="8" t="inlineStr"/>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>Paramètres modifiables dans les préférences mais ne modifie pas dans le logiciel. Ajout d'un bouton "Valider" pour être sûr d'envoyer la commande au logiciel. Le bouton "Remettre à zéro" a validé les modifications au lieu de remettre à zéro.</t>
+        </is>
+      </c>
+      <c r="J10" s="20" t="inlineStr">
+        <is>
+          <t>Corrigé : bouton « Valider » (applique tout de suite aux onglets et lecteurs ouverts), « Annuler », « Valeurs d'usine » par rubrique. « Remettre à zéro maintenant » renommé « Vider l'état de travail » : il vide les destinations et dossiers en cours, pas les Préférences. À refaire dans le nouveau build.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -861,14 +993,25 @@
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr"/>
-      <c r="H11" s="7" t="n"/>
-      <c r="I11" s="8" t="inlineStr"/>
-    </row>
-    <row r="12">
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>RAS</t>
+        </is>
+      </c>
+      <c r="J11" s="19" t="inlineStr"/>
+    </row>
+    <row r="12" ht="25.5" customHeight="1">
       <c r="A12" s="4" t="n">
         <v>8</v>
       </c>
@@ -894,14 +1037,25 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr"/>
-      <c r="H12" s="7" t="n"/>
-      <c r="I12" s="8" t="inlineStr"/>
-    </row>
-    <row r="13">
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>RAS</t>
+        </is>
+      </c>
+      <c r="J12" s="19" t="inlineStr"/>
+    </row>
+    <row r="13" ht="25.5" customHeight="1">
       <c r="A13" s="4" t="n">
         <v>9</v>
       </c>
@@ -927,14 +1081,25 @@
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr"/>
-      <c r="H13" s="7" t="n"/>
-      <c r="I13" s="8" t="inlineStr"/>
-    </row>
-    <row r="14">
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>RAS</t>
+        </is>
+      </c>
+      <c r="J13" s="19" t="inlineStr"/>
+    </row>
+    <row r="14" ht="38.25" customHeight="1">
       <c r="A14" s="4" t="n">
         <v>10</v>
       </c>
@@ -950,12 +1115,12 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Modèle d'arborescence {date}/{camera}/{bobine}. Si un dossier a gardé la structure d'une carte (PRIVATE/M4ROOT, clips A001C001...), le choisir comme source.</t>
+          <t>Reconnaissance de carte : choisir comme source un dossier qui a gardé la structure d'une carte caméra (dossier PRIVATE/M4ROOT de Sony, fichiers .R3D de RED, clips A001C001... d'ARRI). Puis modèle d'arborescence {date}/{camera}/{bobine} et lecture de l'aperçu du chemin.</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Aperçu du chemin cohérent ; « Carte reconnue » affiché sous la source si la structure est celle d'une carte.</t>
+          <t>Sous la source : « Carte reconnue : &lt;type&gt;, bobine &lt;nom&gt; ». L'aperçu du chemin reprend la lettre de caméra et la bobine. Sans structure de carte : rien d'affiché, {bobine} prend le nom du dossier.</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
@@ -963,11 +1128,20 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr"/>
+      <c r="G14" s="6" t="n"/>
       <c r="H14" s="7" t="n"/>
-      <c r="I14" s="8" t="inlineStr"/>
-    </row>
-    <row r="15">
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>Je ne comprends pas ce test?</t>
+        </is>
+      </c>
+      <c r="J14" s="20" t="inlineStr">
+        <is>
+          <t>Test reformulé (colonne Action) : il vérifie que VERIFLOW reconnaît le type de carte d'après ses dossiers. Sans carte caméra, ou sans dossier qui a gardé la structure d'origine, marque « Non testable » et vérifie seulement l'aperçu du chemin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="38.25" customHeight="1">
       <c r="A15" s="4" t="n">
         <v>11</v>
       </c>
@@ -993,14 +1167,29 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr"/>
-      <c r="H15" s="7" t="n"/>
-      <c r="I15" s="8" t="inlineStr"/>
-    </row>
-    <row r="16">
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Source non éjectée car marquée comme utilisée (disque dur externe en USB)</t>
+        </is>
+      </c>
+      <c r="J15" s="20" t="inlineStr">
+        <is>
+          <t>Corrigé à vérifier : VERIFLOW quitte le dossier du disque avant l'éjection (cause probable : le sélecteur de fichiers « Parcourir »). En cas de refus, le message reprend le programme bloquant noté par Windows. Note le message exact s'il revient.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="25.5" customHeight="1">
       <c r="A16" s="4" t="n">
         <v>12</v>
       </c>
@@ -1026,14 +1215,25 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr"/>
-      <c r="H16" s="7" t="n"/>
-      <c r="I16" s="8" t="inlineStr"/>
-    </row>
-    <row r="17">
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>RAS</t>
+        </is>
+      </c>
+      <c r="J16" s="19" t="inlineStr"/>
+    </row>
+    <row r="17" ht="25.5" customHeight="1">
       <c r="A17" s="4" t="n">
         <v>13</v>
       </c>
@@ -1059,14 +1259,29 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr"/>
-      <c r="H17" s="7" t="n"/>
-      <c r="I17" s="8" t="inlineStr"/>
-    </row>
-    <row r="18">
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Non testable</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>Cf point 11</t>
+        </is>
+      </c>
+      <c r="J17" s="20" t="inlineStr">
+        <is>
+          <t>À refaire après le test 11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="25.5" customHeight="1">
       <c r="A18" s="4" t="n">
         <v>14</v>
       </c>
@@ -1095,11 +1310,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr"/>
+      <c r="G18" s="6" t="n"/>
       <c r="H18" s="7" t="n"/>
-      <c r="I18" s="8" t="inlineStr"/>
-    </row>
-    <row r="19">
+      <c r="I18" s="8" t="n"/>
+      <c r="J18" s="19" t="inlineStr"/>
+    </row>
+    <row r="19" ht="25.5" customHeight="1">
       <c r="A19" s="4" t="n">
         <v>15</v>
       </c>
@@ -1128,11 +1344,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr"/>
+      <c r="G19" s="6" t="n"/>
       <c r="H19" s="7" t="n"/>
-      <c r="I19" s="8" t="inlineStr"/>
-    </row>
-    <row r="20">
+      <c r="I19" s="8" t="n"/>
+      <c r="J19" s="19" t="inlineStr"/>
+    </row>
+    <row r="20" ht="38.25" customHeight="1">
       <c r="A20" s="4" t="n">
         <v>16</v>
       </c>
@@ -1161,11 +1378,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr"/>
+      <c r="G20" s="6" t="n"/>
       <c r="H20" s="7" t="n"/>
-      <c r="I20" s="8" t="inlineStr"/>
-    </row>
-    <row r="21">
+      <c r="I20" s="8" t="n"/>
+      <c r="J20" s="19" t="inlineStr"/>
+    </row>
+    <row r="21" ht="25.5" customHeight="1">
       <c r="A21" s="4" t="n">
         <v>17</v>
       </c>
@@ -1194,11 +1412,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr"/>
+      <c r="G21" s="6" t="n"/>
       <c r="H21" s="7" t="n"/>
-      <c r="I21" s="8" t="inlineStr"/>
-    </row>
-    <row r="22">
+      <c r="I21" s="8" t="n"/>
+      <c r="J21" s="19" t="inlineStr"/>
+    </row>
+    <row r="22" ht="38.25" customHeight="1">
       <c r="A22" s="4" t="n">
         <v>18</v>
       </c>
@@ -1227,11 +1446,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr"/>
+      <c r="G22" s="6" t="n"/>
       <c r="H22" s="7" t="n"/>
-      <c r="I22" s="8" t="inlineStr"/>
-    </row>
-    <row r="23">
+      <c r="I22" s="8" t="n"/>
+      <c r="J22" s="19" t="inlineStr"/>
+    </row>
+    <row r="23" ht="25.5" customHeight="1">
       <c r="A23" s="4" t="n">
         <v>19</v>
       </c>
@@ -1260,11 +1480,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr"/>
+      <c r="G23" s="6" t="n"/>
       <c r="H23" s="7" t="n"/>
-      <c r="I23" s="8" t="inlineStr"/>
-    </row>
-    <row r="24">
+      <c r="I23" s="8" t="n"/>
+      <c r="J23" s="19" t="inlineStr"/>
+    </row>
+    <row r="24" ht="38.25" customHeight="1">
       <c r="A24" s="4" t="n">
         <v>20</v>
       </c>
@@ -1293,11 +1514,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr"/>
+      <c r="G24" s="6" t="n"/>
       <c r="H24" s="7" t="n"/>
-      <c r="I24" s="8" t="inlineStr"/>
-    </row>
-    <row r="25">
+      <c r="I24" s="8" t="n"/>
+      <c r="J24" s="19" t="inlineStr"/>
+    </row>
+    <row r="25" ht="25.5" customHeight="1">
       <c r="A25" s="4" t="n">
         <v>21</v>
       </c>
@@ -1326,11 +1548,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr"/>
+      <c r="G25" s="6" t="n"/>
       <c r="H25" s="7" t="n"/>
-      <c r="I25" s="8" t="inlineStr"/>
-    </row>
-    <row r="26">
+      <c r="I25" s="8" t="n"/>
+      <c r="J25" s="19" t="inlineStr"/>
+    </row>
+    <row r="26" ht="25.5" customHeight="1">
       <c r="A26" s="4" t="n">
         <v>22</v>
       </c>
@@ -1359,9 +1582,10 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="G26" s="6" t="inlineStr"/>
+      <c r="G26" s="6" t="n"/>
       <c r="H26" s="7" t="n"/>
-      <c r="I26" s="8" t="inlineStr"/>
+      <c r="I26" s="8" t="n"/>
+      <c r="J26" s="19" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -1392,9 +1616,10 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="G27" s="6" t="inlineStr"/>
+      <c r="G27" s="6" t="n"/>
       <c r="H27" s="7" t="n"/>
-      <c r="I27" s="8" t="inlineStr"/>
+      <c r="I27" s="8" t="n"/>
+      <c r="J27" s="19" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
@@ -1425,9 +1650,10 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr"/>
+      <c r="G28" s="6" t="n"/>
       <c r="H28" s="7" t="n"/>
-      <c r="I28" s="8" t="inlineStr"/>
+      <c r="I28" s="8" t="n"/>
+      <c r="J28" s="19" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
@@ -1458,11 +1684,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="G29" s="6" t="inlineStr"/>
+      <c r="G29" s="6" t="n"/>
       <c r="H29" s="7" t="n"/>
-      <c r="I29" s="8" t="inlineStr"/>
-    </row>
-    <row r="30">
+      <c r="I29" s="8" t="n"/>
+      <c r="J29" s="19" t="inlineStr"/>
+    </row>
+    <row r="30" ht="38.25" customHeight="1">
       <c r="A30" s="4" t="n">
         <v>26</v>
       </c>
@@ -1491,11 +1718,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="G30" s="6" t="inlineStr"/>
+      <c r="G30" s="6" t="n"/>
       <c r="H30" s="7" t="n"/>
-      <c r="I30" s="8" t="inlineStr"/>
-    </row>
-    <row r="31">
+      <c r="I30" s="8" t="n"/>
+      <c r="J30" s="19" t="inlineStr"/>
+    </row>
+    <row r="31" ht="38.25" customHeight="1">
       <c r="A31" s="4" t="n">
         <v>27</v>
       </c>
@@ -1524,11 +1752,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="G31" s="6" t="inlineStr"/>
+      <c r="G31" s="6" t="n"/>
       <c r="H31" s="7" t="n"/>
-      <c r="I31" s="8" t="inlineStr"/>
-    </row>
-    <row r="32">
+      <c r="I31" s="8" t="n"/>
+      <c r="J31" s="19" t="inlineStr"/>
+    </row>
+    <row r="32" ht="25.5" customHeight="1">
       <c r="A32" s="4" t="n">
         <v>28</v>
       </c>
@@ -1557,11 +1786,12 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="G32" s="6" t="inlineStr"/>
+      <c r="G32" s="6" t="n"/>
       <c r="H32" s="7" t="n"/>
-      <c r="I32" s="8" t="inlineStr"/>
-    </row>
-    <row r="33">
+      <c r="I32" s="8" t="n"/>
+      <c r="J32" s="19" t="inlineStr"/>
+    </row>
+    <row r="33" ht="25.5" customHeight="1">
       <c r="A33" s="4" t="n">
         <v>29</v>
       </c>
@@ -1590,23 +1820,24 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="G33" s="6" t="inlineStr"/>
+      <c r="G33" s="6" t="n"/>
       <c r="H33" s="7" t="n"/>
-      <c r="I33" s="8" t="inlineStr"/>
+      <c r="I33" s="8" t="n"/>
+      <c r="J33" s="19" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I33"/>
+  <autoFilter ref="A4:J33"/>
   <conditionalFormatting sqref="G5:G33">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="1">
       <formula>"OK"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="0">
       <formula>"KO"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="3">
       <formula>"Partiel"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="2">
       <formula>"Non testable"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1622,7 +1853,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>
 </file>
 
@@ -1633,19 +1864,17 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="4" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="7" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="16.5" customHeight="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Synthèse (calculée automatiquement depuis l'onglet Tests)</t>
@@ -2442,10 +2671,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="H4:H23">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="1">
       <formula>"Validée"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="0">
       <formula>"À corriger"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2460,17 +2689,15 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="90" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="3" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="16.5" customHeight="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Mode d'emploi</t>
@@ -2501,7 +2728,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="25.5" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
           <t>Résultat</t>
@@ -2525,7 +2752,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="25.5" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
           <t>Commentaires</t>
@@ -2573,7 +2800,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="16.5" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Exemple de ligne remplie</t>
@@ -2612,7 +2839,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="25.5" customHeight="1">
       <c r="A13" s="17" t="n">
         <v>13</v>
       </c>

</xml_diff>

<commit_message>
Recette : retours du 24/10, tests réécrits pas à pas et 8 nouveaux tests
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MoqekrFvgrWkuAe5NHnE5A
</commit_message>
<xml_diff>
--- a/docs/recette/RECETTE_PR_17-37.xlsx
+++ b/docs/recette/RECETTE_PR_17-37.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Légende" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tests'!$A$4:$J$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tests'!$A$4:$J$41</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Tests'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -20,8 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="11">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
+  </numFmts>
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -79,10 +81,26 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -106,7 +124,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
+        <fgColor rgb="FF1F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -114,13 +137,43 @@
         <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -156,7 +209,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -206,11 +259,42 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="10">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -250,6 +334,34 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00D9D9D9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -615,7 +727,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -632,7 +744,7 @@
     <row r="1" ht="18" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Recette VERIFLOW : PR 17 à 37 (build de la branche claude/recette, Windows 11)</t>
+          <t>Recette VERIFLOW : PR 17 à 38 (build de la branche claude/recette, Windows 11)</t>
         </is>
       </c>
     </row>
@@ -691,7 +803,7 @@
       </c>
       <c r="J4" s="18" t="inlineStr">
         <is>
-          <t>Réponse de Claude (23/10)</t>
+          <t>Réponse de Claude (mise à jour 25/10)</t>
         </is>
       </c>
     </row>
@@ -737,7 +849,7 @@
           <t>RAS</t>
         </is>
       </c>
-      <c r="J5" s="19" t="inlineStr"/>
+      <c r="J5" s="19" t="n"/>
     </row>
     <row r="6" ht="25.5" customHeight="1">
       <c r="A6" s="4" t="n">
@@ -781,7 +893,7 @@
           <t>RAS</t>
         </is>
       </c>
-      <c r="J6" s="19" t="inlineStr"/>
+      <c r="J6" s="19" t="n"/>
     </row>
     <row r="7" ht="25.5" customHeight="1">
       <c r="A7" s="4" t="n">
@@ -825,7 +937,7 @@
           <t>RAS</t>
         </is>
       </c>
-      <c r="J7" s="19" t="inlineStr"/>
+      <c r="J7" s="19" t="n"/>
     </row>
     <row r="8" ht="25.5" customHeight="1">
       <c r="A8" s="4" t="n">
@@ -862,16 +974,16 @@
         </is>
       </c>
       <c r="H8" s="7" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>Manuel assez sommaire, il faut le développer plus pour permettre l'utilisateur d'être autonome sur le logiciel</t>
-        </is>
-      </c>
-      <c r="J8" s="20" t="inlineStr">
-        <is>
-          <t>Guide développé : 12 chapitres au lieu de 7, 610 lignes au lieu de 194 (journée de tournage, recettes TRANSCODE, problèmes fréquents, glossaire). À relire dans le nouveau build.</t>
+          <t>Ajouter des images du logiciel avec mise en avant des points mentionnés</t>
+        </is>
+      </c>
+      <c r="J8" s="21" t="inlineStr">
+        <is>
+          <t>Captures du guide avec les points mis en évidence : à faire (PR à venir).</t>
         </is>
       </c>
     </row>
@@ -917,7 +1029,7 @@
           <t>RAS</t>
         </is>
       </c>
-      <c r="J9" s="19" t="inlineStr"/>
+      <c r="J9" s="19" t="n"/>
     </row>
     <row r="10" ht="63.75" customHeight="1">
       <c r="A10" s="4" t="n">
@@ -950,7 +1062,7 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Partiel</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="H10" s="7" t="n">
@@ -958,7 +1070,7 @@
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>Paramètres modifiables dans les préférences mais ne modifie pas dans le logiciel. Ajout d'un bouton "Valider" pour être sûr d'envoyer la commande au logiciel. Le bouton "Remettre à zéro" a validé les modifications au lieu de remettre à zéro.</t>
+          <t>RAS</t>
         </is>
       </c>
       <c r="J10" s="20" t="inlineStr">
@@ -1009,7 +1121,7 @@
           <t>RAS</t>
         </is>
       </c>
-      <c r="J11" s="19" t="inlineStr"/>
+      <c r="J11" s="19" t="n"/>
     </row>
     <row r="12" ht="25.5" customHeight="1">
       <c r="A12" s="4" t="n">
@@ -1053,7 +1165,7 @@
           <t>RAS</t>
         </is>
       </c>
-      <c r="J12" s="19" t="inlineStr"/>
+      <c r="J12" s="19" t="n"/>
     </row>
     <row r="13" ht="25.5" customHeight="1">
       <c r="A13" s="4" t="n">
@@ -1097,7 +1209,7 @@
           <t>RAS</t>
         </is>
       </c>
-      <c r="J13" s="19" t="inlineStr"/>
+      <c r="J13" s="19" t="n"/>
     </row>
     <row r="14" ht="38.25" customHeight="1">
       <c r="A14" s="4" t="n">
@@ -1125,14 +1237,20 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="n"/>
-      <c r="H14" s="7" t="n"/>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>46318</v>
+      </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>Je ne comprends pas ce test?</t>
+          <t>RAS</t>
         </is>
       </c>
       <c r="J14" s="20" t="inlineStr">
@@ -1172,7 +1290,7 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Partiel</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
@@ -1180,12 +1298,12 @@
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
-          <t>Source non éjectée car marquée comme utilisée (disque dur externe en USB)</t>
-        </is>
-      </c>
-      <c r="J15" s="20" t="inlineStr">
-        <is>
-          <t>Corrigé à vérifier. Ton journal Windows (Kernel-PnP 225 du 18/10) désignait VERIFLOW, et rien le 22/10 : la commande « Éjecter » de l'Explorateur n'agissait sans doute pas sur un disque dur USB. VERIFLOW éjecte maintenant comme « Retirer le périphérique en toute sécurité », après avoir quitté le disque. En cas de refus, le message donne la raison de Windows : note-le ici.</t>
+          <t>Dans l'explorer de Veriflow, il y a un icone "ejecter" à côté des disques externes, cartes…etc, il faudrait que cet icône permette aussi d'éjecter ces supports en toute sécurité</t>
+        </is>
+      </c>
+      <c r="J15" s="21" t="inlineStr">
+        <is>
+          <t>Bouton ⏏ de l'explorateur : fait, voir test 30 (build du 24/10 (run 40104706786)).</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1349,7 @@
           <t>RAS</t>
         </is>
       </c>
-      <c r="J16" s="19" t="inlineStr"/>
+      <c r="J16" s="19" t="n"/>
     </row>
     <row r="17" ht="25.5" customHeight="1">
       <c r="A17" s="4" t="n">
@@ -1264,7 +1382,7 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Non testable</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -1272,7 +1390,7 @@
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>Cf point 11</t>
+          <t>RAS</t>
         </is>
       </c>
       <c r="J17" s="20" t="inlineStr">
@@ -1281,7 +1399,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="25.5" customHeight="1">
+    <row r="18" ht="63.75" customHeight="1">
       <c r="A18" s="4" t="n">
         <v>14</v>
       </c>
@@ -1307,13 +1425,27 @@
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="n"/>
-      <c r="H18" s="7" t="n"/>
-      <c r="I18" s="8" t="n"/>
-      <c r="J18" s="19" t="inlineStr"/>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="n">
+        <v>46319</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Fenêtre glissée sur le 2e écran, double clic dans la barre du haut pour adapter à la taille de l'écran (pas en plein écran, juste fenêtre adaptée). Echap, ferme le lecteur pop-up. Double clic sur le même rush, le lecteur pop-up se rouvre sur le 1er écran, pas sur le 2e</t>
+        </is>
+      </c>
+      <c r="J18" s="21" t="inlineStr">
+        <is>
+          <t>Corrigé : place mémorisée en pixels réels et fenêtre agrandie rétablie sur le même écran. À refaire avec le build du 24/10 (run 40104706786).</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="25.5" customHeight="1">
       <c r="A19" s="4" t="n">
@@ -1341,15 +1473,25 @@
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="n"/>
-      <c r="H19" s="7" t="n"/>
-      <c r="I19" s="8" t="n"/>
-      <c r="J19" s="19" t="inlineStr"/>
-    </row>
-    <row r="20" ht="38.25" customHeight="1">
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="n">
+        <v>46319</v>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>Même protocole, pas en plein écran, juste fenêtre adaptée, la fenêtre reste bien en place et lance le 2e rush</t>
+        </is>
+      </c>
+      <c r="J19" s="19" t="n"/>
+    </row>
+    <row r="20" ht="63.75" customHeight="1">
       <c r="A20" s="4" t="n">
         <v>16</v>
       </c>
@@ -1375,15 +1517,29 @@
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G20" s="6" t="n"/>
-      <c r="H20" s="7" t="n"/>
-      <c r="I20" s="8" t="n"/>
-      <c r="J20" s="19" t="inlineStr"/>
-    </row>
-    <row r="21" ht="25.5" customHeight="1">
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="n">
+        <v>46319</v>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>Lecteur pop-up déplacé sur le 2e écran, sortie TV choisie, affichage plein écran. Curseur souris disparait au bout de 2 sec et réapparait si je le bouge, mais de contrôle de lecture possible avec espace : le contrôle est resté sur le choix du moniteur !</t>
+        </is>
+      </c>
+      <c r="J20" s="21" t="inlineStr">
+        <is>
+          <t>Corrigé : après le choix du moniteur, le clavier revient au lecteur (Espace, J/K/L). À refaire avec le build du 24/10 (run 40104706786).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="63.75" customHeight="1">
       <c r="A21" s="4" t="n">
         <v>17</v>
       </c>
@@ -1409,15 +1565,29 @@
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="n"/>
-      <c r="H21" s="7" t="n"/>
-      <c r="I21" s="8" t="n"/>
-      <c r="J21" s="19" t="inlineStr"/>
-    </row>
-    <row r="22" ht="38.25" customHeight="1">
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="n">
+        <v>46319</v>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Lecteur pop-up ouvert sur le 2e écran. Je débranche le 2e écran, le lecteur revient sur l'écran principal. Je ferme le lecteur pop-up, je double clic sur un rush, le lecteur pop-up s'ouvre sur l'écran principal (toujours pas de 2e écran branché) mais message d'erreur audio (voir capture)</t>
+        </is>
+      </c>
+      <c r="J21" s="21" t="inlineStr">
+        <is>
+          <t>Corrigé : la carte son est ouverte sur un fil neuf (erreur « mode thread » de Windows). À refaire avec le build du 24/10 (run 40104706786).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="127.5" customHeight="1">
       <c r="A22" s="4" t="n">
         <v>18</v>
       </c>
@@ -1443,13 +1613,28 @@
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G22" s="6" t="n"/>
-      <c r="H22" s="7" t="n"/>
-      <c r="I22" s="8" t="n"/>
-      <c r="J22" s="19" t="inlineStr"/>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="n">
+        <v>46319</v>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>Test sur média plus petit, player pop-up, le son arrive au bout de quelques secondes après le début de lecture.
+Metadata : l'enregistrement des modif ne se fait que par un clic sur le bouton enregistrer, il faut ajouter la validation par la touche Return et la touche entrée du pavé numérique du clavier + bouton enregistrer superposé à la colonne de manière non esthétique. Dans la fenêtre centrale, le TC n'est pas affiché. (voir capture) + impossible de redimenssioner les colonnes à la main ni changer qeulle colonne sont visible/invisible</t>
+        </is>
+      </c>
+      <c r="J22" s="21" t="inlineStr">
+        <is>
+          <t>Corrigé : Entrée (clavier et pavé numérique), barre Enregistrer, TC des WAV : voir test 34. Son en retard : à revérifier avec le build du 24/10 (run 40104706786) (peut venir de l'erreur audio du test 17). Colonnes réglables et masquables : à faire (PR à venir).</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="25.5" customHeight="1">
       <c r="A23" s="4" t="n">
@@ -1483,9 +1668,9 @@
       <c r="G23" s="6" t="n"/>
       <c r="H23" s="7" t="n"/>
       <c r="I23" s="8" t="n"/>
-      <c r="J23" s="19" t="inlineStr"/>
-    </row>
-    <row r="24" ht="38.25" customHeight="1">
+      <c r="J23" s="19" t="n"/>
+    </row>
+    <row r="24" ht="153" customHeight="1">
       <c r="A24" s="4" t="n">
         <v>20</v>
       </c>
@@ -1501,23 +1686,39 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Cocher Préférences &gt; PLAYER &gt; « Ouvrir la saisie du rapport à chaque nouvelle prise », ouvrir un projet, charger plusieurs prises, puis recharger la même.</t>
+          <t>1. Préférences &gt; PLAYER : cocher « Ouvrir la saisie du rapport à chaque nouvelle prise », puis Valider. 2. Ouvrir un projet. 3. Dans MEDIA, ouvrir un clip dans le PLAYER. 4. Fermer la saisie (Échap), ouvrir un AUTRE clip dans le PLAYER. 5. Rouvrir le MÊME clip.</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Saisie ouverte à chaque nouvelle prise ; pas en rechargeant la même.</t>
+          <t>Étape 3 et 4 : la fenêtre de saisie du rapport (touche R) s'ouvre seule. Étape 5 : elle ne s'ouvre pas.</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="n"/>
-      <c r="H24" s="7" t="n"/>
-      <c r="I24" s="8" t="n"/>
-      <c r="J24" s="19" t="inlineStr"/>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="n">
+        <v>46319</v>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Création d'un projet, nom du projet pas centré sur le haut de la fenêtre. Case cochée dans les préférences. Je n'ai pas compris la suite du protocole. Explique moi pas à pas.
+J'ai essayé d'ouvrir plusieurs rushes audio dans l'onglet PLAYER : ils sont tous ouverts en même temps et l'affichage de l'application s'est décalé. Pour pouvoir lire plusieurs rushes dans PLAYER, il faut créer un système de liste de lecture.
+Dans les consles audio du PLAYER, le clic sur les boutons SOLO et/ou MUTE ne fais que noircir le bouton, il faut qu'il passe en couleur pour le mettre en évidence.</t>
+        </is>
+      </c>
+      <c r="J24" s="21" t="inlineStr">
+        <is>
+          <t>Test réécrit pas à pas (colonne Action). Projet centré et SOLO/MUTE : voir tests 32 et 33. Liste de lecture du PLAYER : à faire (PR à venir).</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="25.5" customHeight="1">
       <c r="A25" s="4" t="n">
@@ -1545,13 +1746,23 @@
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="n"/>
-      <c r="H25" s="7" t="n"/>
-      <c r="I25" s="8" t="n"/>
-      <c r="J25" s="19" t="inlineStr"/>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="n">
+        <v>46319</v>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>RAS</t>
+        </is>
+      </c>
+      <c r="J25" s="19" t="n"/>
     </row>
     <row r="26" ht="25.5" customHeight="1">
       <c r="A26" s="4" t="n">
@@ -1585,7 +1796,7 @@
       <c r="G26" s="6" t="n"/>
       <c r="H26" s="7" t="n"/>
       <c r="I26" s="8" t="n"/>
-      <c r="J26" s="19" t="inlineStr"/>
+      <c r="J26" s="19" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -1619,9 +1830,9 @@
       <c r="G27" s="6" t="n"/>
       <c r="H27" s="7" t="n"/>
       <c r="I27" s="8" t="n"/>
-      <c r="J27" s="19" t="inlineStr"/>
-    </row>
-    <row r="28">
+      <c r="J27" s="19" t="n"/>
+    </row>
+    <row r="28" ht="51" customHeight="1">
       <c r="A28" s="4" t="n">
         <v>24</v>
       </c>
@@ -1647,13 +1858,27 @@
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="n"/>
-      <c r="H28" s="7" t="n"/>
-      <c r="I28" s="8" t="n"/>
-      <c r="J28" s="19" t="inlineStr"/>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="n">
+        <v>46319</v>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>Mode AUDIO : pas de choix du dossier pour les fichier resynchro - direct dans le dossier des rushes vidéo. Fichiers resynchro ouvert dans Resolve : que de l'audio, pas de vidéo.</t>
+        </is>
+      </c>
+      <c r="J28" s="21" t="inlineStr">
+        <is>
+          <t>Image absente dans Resolve : limite de Resolve gratuit (H.264 10 bits 4:2:2), lu dans Premiere. Mauvais son : corrigé, voir tests 35 à 37. Choix du dossier en mode AUDIO : envoie-moi une capture de la colonne de droite si le problème revient.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
@@ -1681,13 +1906,23 @@
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G29" s="6" t="n"/>
-      <c r="H29" s="7" t="n"/>
-      <c r="I29" s="8" t="n"/>
-      <c r="J29" s="19" t="inlineStr"/>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="n">
+        <v>46319</v>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>RAS</t>
+        </is>
+      </c>
+      <c r="J29" s="19" t="n"/>
     </row>
     <row r="30" ht="38.25" customHeight="1">
       <c r="A30" s="4" t="n">
@@ -1705,12 +1940,12 @@
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Exporter de Resolve un titre avec transparence en ProRes 4444 ; le convertir dans VERIFLOW en ProRes 4444 puis en PNG ; réimporter dans Resolve.</t>
+          <t>1. Resolve : titre (texte blanc) sur une timeline vide. 2. Deliver : QuickTime, Apple ProRes 4444, « Export Alpha » coché. 3. TRANSCODE : ajouter ce fichier, préréglage ProRes 4444, lancer. 4. Refaire avec le préréglage PNG. 5. Réimporter les deux dans Resolve, au-dessus d'une image.</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>Transparence conservée dans les deux cas.</t>
+          <t>Le texte est détouré sur l'image (fond transparent). Fond noir = transparence perdue.</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
@@ -1720,8 +1955,16 @@
       </c>
       <c r="G30" s="6" t="n"/>
       <c r="H30" s="7" t="n"/>
-      <c r="I30" s="8" t="n"/>
-      <c r="J30" s="19" t="inlineStr"/>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>Je ne comprends pas, explique pas à pas</t>
+        </is>
+      </c>
+      <c r="J30" s="21" t="inlineStr">
+        <is>
+          <t>Test réécrit pas à pas (colonne Action).</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="38.25" customHeight="1">
       <c r="A31" s="4" t="n">
@@ -1739,12 +1982,12 @@
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Ouvrir un ASS (Aegisub, ou un SRT enregistré en ASS) ; corriger un texte et un temps ; enregistrer ; rouvrir ; incruster dans une vidéo avec TRANSCODE.</t>
+          <t>1. TRANSCODE &gt; Incrustations : « Créer des sous-titres », saisir deux sous-titres, enregistrer en ASS. 2. Rouvrir ce fichier avec « Éditer », corriger un texte et un temps, enregistrer. 3. Cocher l'incrustation de ce fichier sur une vidéo et lancer. 4. (Si Aegisub) ouvrir le fichier.</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Styles intacts à la réouverture ; styles respectés à l'image.</t>
+          <t>Corrections conservées à la réouverture ; sous-titres visibles à l'image aux bons temps ; styles intacts dans Aegisub.</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
@@ -1754,8 +1997,16 @@
       </c>
       <c r="G31" s="6" t="n"/>
       <c r="H31" s="7" t="n"/>
-      <c r="I31" s="8" t="n"/>
-      <c r="J31" s="19" t="inlineStr"/>
+      <c r="I31" s="8" t="inlineStr">
+        <is>
+          <t>Je ne comprends pas, explique pas à pas</t>
+        </is>
+      </c>
+      <c r="J31" s="21" t="inlineStr">
+        <is>
+          <t>Test réécrit pas à pas (colonne Action).</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="25.5" customHeight="1">
       <c r="A32" s="4" t="n">
@@ -1773,25 +2024,39 @@
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Préférences &gt; Général &gt; « Repartir à zéro », fermer puis rouvrir VERIFLOW.</t>
+          <t>Préférences &gt; Général &gt; liste « À l'ouverture de VERIFLOW » : choisir « Repartir à zéro ». Fermer puis rouvrir VERIFLOW.</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>État de travail vide ; langue et favoris conservés.</t>
+          <t>État de travail vide (destinations, dossiers dépliés) ; langue et favoris conservés.</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G32" s="6" t="n"/>
-      <c r="H32" s="7" t="n"/>
-      <c r="I32" s="8" t="n"/>
-      <c r="J32" s="19" t="inlineStr"/>
-    </row>
-    <row r="33" ht="25.5" customHeight="1">
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>Non testable</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="n">
+        <v>46319</v>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>Il n'y a plus l'option "repartir de zéro", seulement "vider l'état de travail" ou "Effacer toutes les données"</t>
+        </is>
+      </c>
+      <c r="J32" s="21" t="inlineStr">
+        <is>
+          <t>L'option est dans la liste déroulante « À l'ouverture de VERIFLOW » (Préférences &gt; Général), au-dessus des deux boutons. À refaire.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="38.25" customHeight="1">
       <c r="A33" s="4" t="n">
         <v>29</v>
       </c>
@@ -1817,38 +2082,356 @@
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="n">
+        <v>46319</v>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>Il faut que l'install se fasse dans le dossier Programme et non dans le dossier AppData (voir capture). Sinon, logiciel bien réintsallé à zéro.</t>
+        </is>
+      </c>
+      <c r="J33" s="21" t="inlineStr">
+        <is>
+          <t>Corrigé : installation dans C:\Program Files\VERIFLOW (droits administrateur demandés). Désinstalle d'abord l'ancienne version (AppData). À refaire avec le build du 24/10 (run 40104706786).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="22" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="23" t="inlineStr">
+        <is>
+          <t>B. OFFLOAD</t>
+        </is>
+      </c>
+      <c r="C34" s="22" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D34" s="23" t="inlineStr">
+        <is>
+          <t>Explorateur : cliquer sur le bouton ⏏ à côté d'un disque externe ou d'une carte.</t>
+        </is>
+      </c>
+      <c r="E34" s="23" t="inlineStr">
+        <is>
+          <t>Barre d'état : « Éjecté, tu peux le débrancher ». Le disque disparaît de l'explorateur. En cas de refus, le message donne la raison de Windows.</t>
+        </is>
+      </c>
+      <c r="F34" s="24" t="inlineStr">
+        <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="G33" s="6" t="n"/>
-      <c r="H33" s="7" t="n"/>
-      <c r="I33" s="8" t="n"/>
-      <c r="J33" s="19" t="inlineStr"/>
+      <c r="G34" s="24" t="inlineStr"/>
+      <c r="H34" s="25" t="n"/>
+      <c r="I34" s="26" t="inlineStr"/>
+      <c r="J34" s="27" t="inlineStr">
+        <is>
+          <t>Nouveau test (correctifs du 24/10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="22" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="23" t="inlineStr">
+        <is>
+          <t>B. OFFLOAD</t>
+        </is>
+      </c>
+      <c r="C35" s="22" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D35" s="23" t="inlineStr">
+        <is>
+          <t>Explorateur : déplier le disque HERVE EDU (F:).</t>
+        </is>
+      </c>
+      <c r="E35" s="23" t="inlineStr">
+        <is>
+          <t>Les dossiers FOUND.000 à FOUND.004 n'apparaissent plus.</t>
+        </is>
+      </c>
+      <c r="F35" s="24" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="G35" s="24" t="inlineStr"/>
+      <c r="H35" s="25" t="n"/>
+      <c r="I35" s="26" t="inlineStr"/>
+      <c r="J35" s="27" t="inlineStr">
+        <is>
+          <t>Nouveau test (correctifs du 24/10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="22" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="23" t="inlineStr">
+        <is>
+          <t>D. PLAYER</t>
+        </is>
+      </c>
+      <c r="C36" s="22" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="D36" s="23" t="inlineStr">
+        <is>
+          <t>PLAYER en mode AUDIO : cliquer SOLO puis MUTE sur une piste.</t>
+        </is>
+      </c>
+      <c r="E36" s="23" t="inlineStr">
+        <is>
+          <t>SOLO en orange, MUTE en rouge quand ils sont actifs.</t>
+        </is>
+      </c>
+      <c r="F36" s="24" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="G36" s="24" t="inlineStr"/>
+      <c r="H36" s="25" t="n"/>
+      <c r="I36" s="26" t="inlineStr"/>
+      <c r="J36" s="27" t="inlineStr">
+        <is>
+          <t>Nouveau test (correctifs du 24/10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="22" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="23" t="inlineStr">
+        <is>
+          <t>A. Installation et menus</t>
+        </is>
+      </c>
+      <c r="C37" s="22" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="D37" s="23" t="inlineStr">
+        <is>
+          <t>Ouvrir un projet et regarder la barre du haut.</t>
+        </is>
+      </c>
+      <c r="E37" s="23" t="inlineStr">
+        <is>
+          <t>Nom du projet au centre de la fenêtre.</t>
+        </is>
+      </c>
+      <c r="F37" s="24" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="G37" s="24" t="inlineStr"/>
+      <c r="H37" s="25" t="n"/>
+      <c r="I37" s="26" t="inlineStr"/>
+      <c r="J37" s="27" t="inlineStr">
+        <is>
+          <t>Nouveau test (correctifs du 24/10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="22" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="23" t="inlineStr">
+        <is>
+          <t>C. MEDIA et second écran</t>
+        </is>
+      </c>
+      <c r="C38" s="22" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="D38" s="23" t="inlineStr">
+        <is>
+          <t>MEDIA : modifier un champ, puis Entrée (clavier principal), puis un autre avec Entrée du pavé numérique. Regarder la barre Enregistrer et la colonne TC en mode AUDIO.</t>
+        </is>
+      </c>
+      <c r="E38" s="23" t="inlineStr">
+        <is>
+          <t>Enregistré à chaque Entrée ; barre Enregistrer sur toute la largeur, séparée des champs ; TC affiché pour les WAV.</t>
+        </is>
+      </c>
+      <c r="F38" s="24" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="G38" s="24" t="inlineStr"/>
+      <c r="H38" s="25" t="n"/>
+      <c r="I38" s="26" t="inlineStr"/>
+      <c r="J38" s="27" t="inlineStr">
+        <is>
+          <t>Nouveau test (correctifs du 24/10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="22" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="23" t="inlineStr">
+        <is>
+          <t>E. SYNC</t>
+        </is>
+      </c>
+      <c r="C39" s="22" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="D39" s="23" t="inlineStr">
+        <is>
+          <t>SYNC : un rush vidéo avec LTC sur une piste et son témoin sur l'autre, avec son WAV. Méthode Automatique, Analyser.</t>
+        </is>
+      </c>
+      <c r="E39" s="23" t="inlineStr">
+        <is>
+          <t>Colonne Méthode : LTC ; badge LTC à côté du timecode ; TC = celui du LTC (pas l'horloge de la Panasonic).</t>
+        </is>
+      </c>
+      <c r="F39" s="24" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="G39" s="24" t="inlineStr"/>
+      <c r="H39" s="25" t="n"/>
+      <c r="I39" s="26" t="inlineStr"/>
+      <c r="J39" s="27" t="inlineStr">
+        <is>
+          <t>Nouveau test (correctifs du 24/10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="22" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="23" t="inlineStr">
+        <is>
+          <t>E. SYNC</t>
+        </is>
+      </c>
+      <c r="C40" s="22" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="D40" s="23" t="inlineStr">
+        <is>
+          <t>SYNC : tous les rushes Panasonic sans LTC et tous les sons (tests compris), méthode Automatique.</t>
+        </is>
+      </c>
+      <c r="E40" s="23" t="inlineStr">
+        <is>
+          <t>Bon son pour chaque plan ; remarque « timecode sans rapport avec le son : son retrouvé par la forme d'onde » ; les sons de test restent non utilisés (mode AUDIO).</t>
+        </is>
+      </c>
+      <c r="F40" s="24" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="G40" s="24" t="inlineStr"/>
+      <c r="H40" s="25" t="n"/>
+      <c r="I40" s="26" t="inlineStr"/>
+      <c r="J40" s="27" t="inlineStr">
+        <is>
+          <t>Nouveau test (correctifs du 24/10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="22" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="23" t="inlineStr">
+        <is>
+          <t>E. SYNC</t>
+        </is>
+      </c>
+      <c r="C41" s="22" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="D41" s="23" t="inlineStr">
+        <is>
+          <t>SYNC : créer les fichiers synchronisés (option « une piste mono par canal » cochée par défaut), puis les ouvrir dans Premiere.</t>
+        </is>
+      </c>
+      <c r="E41" s="23" t="inlineStr">
+        <is>
+          <t>Image présente ; 6 pistes mono de l'enregistreur + pistes caméra ; son calé sur le clap.</t>
+        </is>
+      </c>
+      <c r="F41" s="24" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="G41" s="24" t="inlineStr"/>
+      <c r="H41" s="25" t="n"/>
+      <c r="I41" s="26" t="inlineStr"/>
+      <c r="J41" s="27" t="inlineStr">
+        <is>
+          <t>Nouveau test (correctifs du 24/10).</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J33"/>
-  <conditionalFormatting sqref="G5:G33">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="1">
+  <autoFilter ref="A4:J41"/>
+  <conditionalFormatting sqref="G5:G41">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="6">
       <formula>"OK"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="7">
       <formula>"KO"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="3">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="8">
       <formula>"Partiel"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="9">
       <formula>"Non testable"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="F5:F33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F5:F41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Oui,Non"</formula1>
     </dataValidation>
-    <dataValidation sqref="G5:G33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,KO,Partiel,Non testable"</formula1>
     </dataValidation>
-    <dataValidation sqref="H5:H33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date" operator="greaterThan">
+    <dataValidation sqref="H5:H41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date" operator="greaterThan">
       <formula1>DATE(2026,1,1)</formula1>
     </dataValidation>
   </dataValidations>
@@ -1864,17 +2447,19 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="5"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="8"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1">
+    <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Synthèse (calculée automatiquement depuis l'onglet Tests)</t>
@@ -1882,799 +2467,827 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="28" t="inlineStr">
         <is>
           <t>PR</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="28" t="inlineStr">
         <is>
           <t>Tests</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" s="28" t="inlineStr">
         <is>
           <t>Effectués</t>
         </is>
       </c>
-      <c r="D3" s="10" t="inlineStr">
+      <c r="D3" s="28" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="E3" s="28" t="inlineStr">
         <is>
           <t>KO</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="F3" s="28" t="inlineStr">
         <is>
           <t>Partiel</t>
         </is>
       </c>
-      <c r="G3" s="10" t="inlineStr">
+      <c r="G3" s="28" t="inlineStr">
         <is>
           <t>Non testable</t>
         </is>
       </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="H3" s="28" t="inlineStr">
         <is>
           <t>Statut</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>17</t>
         </is>
       </c>
-      <c r="B4" s="11">
-        <f>COUNTIF(Tests!$C$5:$C$33,"*"&amp;A4&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C4" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A4&amp;"*",Tests!$F$5:$F$33,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D4" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A4&amp;"*",Tests!$G$5:$G$33,"OK")</f>
-        <v/>
-      </c>
-      <c r="E4" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A4&amp;"*",Tests!$G$5:$G$33,"KO")</f>
-        <v/>
-      </c>
-      <c r="F4" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A4&amp;"*",Tests!$G$5:$G$33,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G4" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A4&amp;"*",Tests!$G$5:$G$33,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H4" s="11">
+      <c r="B4" s="29">
+        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A4&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C4" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A4&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D4" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A4&amp;"*",Tests!$G$5:$G$41,"OK")</f>
+        <v/>
+      </c>
+      <c r="E4" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A4&amp;"*",Tests!$G$5:$G$41,"KO")</f>
+        <v/>
+      </c>
+      <c r="F4" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A4&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G4" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A4&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H4" s="29">
         <f>IF(E4&gt;0,"À corriger",IF(D4+G4=B4,"Validée",IF(C4=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="B5" s="11">
-        <f>COUNTIF(Tests!$C$5:$C$33,"*"&amp;A5&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C5" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A5&amp;"*",Tests!$F$5:$F$33,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D5" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A5&amp;"*",Tests!$G$5:$G$33,"OK")</f>
-        <v/>
-      </c>
-      <c r="E5" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A5&amp;"*",Tests!$G$5:$G$33,"KO")</f>
-        <v/>
-      </c>
-      <c r="F5" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A5&amp;"*",Tests!$G$5:$G$33,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G5" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A5&amp;"*",Tests!$G$5:$G$33,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H5" s="11">
+      <c r="B5" s="29">
+        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A5&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C5" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A5&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D5" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A5&amp;"*",Tests!$G$5:$G$41,"OK")</f>
+        <v/>
+      </c>
+      <c r="E5" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A5&amp;"*",Tests!$G$5:$G$41,"KO")</f>
+        <v/>
+      </c>
+      <c r="F5" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A5&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G5" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A5&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H5" s="29">
         <f>IF(E5&gt;0,"À corriger",IF(D5+G5=B5,"Validée",IF(C5=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="29" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="B6" s="11">
-        <f>COUNTIF(Tests!$C$5:$C$33,"*"&amp;A6&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C6" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A6&amp;"*",Tests!$F$5:$F$33,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D6" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A6&amp;"*",Tests!$G$5:$G$33,"OK")</f>
-        <v/>
-      </c>
-      <c r="E6" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A6&amp;"*",Tests!$G$5:$G$33,"KO")</f>
-        <v/>
-      </c>
-      <c r="F6" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A6&amp;"*",Tests!$G$5:$G$33,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G6" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A6&amp;"*",Tests!$G$5:$G$33,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H6" s="11">
+      <c r="B6" s="29">
+        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A6&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C6" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A6&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D6" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A6&amp;"*",Tests!$G$5:$G$41,"OK")</f>
+        <v/>
+      </c>
+      <c r="E6" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A6&amp;"*",Tests!$G$5:$G$41,"KO")</f>
+        <v/>
+      </c>
+      <c r="F6" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A6&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G6" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A6&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H6" s="29">
         <f>IF(E6&gt;0,"À corriger",IF(D6+G6=B6,"Validée",IF(C6=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="29" t="inlineStr">
         <is>
           <t>23</t>
         </is>
       </c>
-      <c r="B7" s="11">
-        <f>COUNTIF(Tests!$C$5:$C$33,"*"&amp;A7&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C7" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A7&amp;"*",Tests!$F$5:$F$33,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D7" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A7&amp;"*",Tests!$G$5:$G$33,"OK")</f>
-        <v/>
-      </c>
-      <c r="E7" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A7&amp;"*",Tests!$G$5:$G$33,"KO")</f>
-        <v/>
-      </c>
-      <c r="F7" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A7&amp;"*",Tests!$G$5:$G$33,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G7" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A7&amp;"*",Tests!$G$5:$G$33,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H7" s="11">
+      <c r="B7" s="29">
+        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A7&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C7" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A7&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D7" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A7&amp;"*",Tests!$G$5:$G$41,"OK")</f>
+        <v/>
+      </c>
+      <c r="E7" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A7&amp;"*",Tests!$G$5:$G$41,"KO")</f>
+        <v/>
+      </c>
+      <c r="F7" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A7&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G7" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A7&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H7" s="29">
         <f>IF(E7&gt;0,"À corriger",IF(D7+G7=B7,"Validée",IF(C7=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="29" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="B8" s="11">
-        <f>COUNTIF(Tests!$C$5:$C$33,"*"&amp;A8&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C8" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A8&amp;"*",Tests!$F$5:$F$33,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D8" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A8&amp;"*",Tests!$G$5:$G$33,"OK")</f>
-        <v/>
-      </c>
-      <c r="E8" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A8&amp;"*",Tests!$G$5:$G$33,"KO")</f>
-        <v/>
-      </c>
-      <c r="F8" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A8&amp;"*",Tests!$G$5:$G$33,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G8" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A8&amp;"*",Tests!$G$5:$G$33,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H8" s="11">
+      <c r="B8" s="29">
+        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A8&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C8" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A8&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D8" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A8&amp;"*",Tests!$G$5:$G$41,"OK")</f>
+        <v/>
+      </c>
+      <c r="E8" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A8&amp;"*",Tests!$G$5:$G$41,"KO")</f>
+        <v/>
+      </c>
+      <c r="F8" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A8&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G8" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A8&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H8" s="29">
         <f>IF(E8&gt;0,"À corriger",IF(D8+G8=B8,"Validée",IF(C8=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="B9" s="11">
-        <f>COUNTIF(Tests!$C$5:$C$33,"*"&amp;A9&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C9" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A9&amp;"*",Tests!$F$5:$F$33,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D9" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A9&amp;"*",Tests!$G$5:$G$33,"OK")</f>
-        <v/>
-      </c>
-      <c r="E9" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A9&amp;"*",Tests!$G$5:$G$33,"KO")</f>
-        <v/>
-      </c>
-      <c r="F9" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A9&amp;"*",Tests!$G$5:$G$33,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G9" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A9&amp;"*",Tests!$G$5:$G$33,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H9" s="11">
+      <c r="B9" s="29">
+        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A9&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C9" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A9&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D9" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A9&amp;"*",Tests!$G$5:$G$41,"OK")</f>
+        <v/>
+      </c>
+      <c r="E9" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A9&amp;"*",Tests!$G$5:$G$41,"KO")</f>
+        <v/>
+      </c>
+      <c r="F9" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A9&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G9" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A9&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H9" s="29">
         <f>IF(E9&gt;0,"À corriger",IF(D9+G9=B9,"Validée",IF(C9=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="29" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="B10" s="11">
-        <f>COUNTIF(Tests!$C$5:$C$33,"*"&amp;A10&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C10" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A10&amp;"*",Tests!$F$5:$F$33,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D10" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A10&amp;"*",Tests!$G$5:$G$33,"OK")</f>
-        <v/>
-      </c>
-      <c r="E10" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A10&amp;"*",Tests!$G$5:$G$33,"KO")</f>
-        <v/>
-      </c>
-      <c r="F10" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A10&amp;"*",Tests!$G$5:$G$33,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G10" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A10&amp;"*",Tests!$G$5:$G$33,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H10" s="11">
+      <c r="B10" s="29">
+        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A10&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C10" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A10&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D10" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A10&amp;"*",Tests!$G$5:$G$41,"OK")</f>
+        <v/>
+      </c>
+      <c r="E10" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A10&amp;"*",Tests!$G$5:$G$41,"KO")</f>
+        <v/>
+      </c>
+      <c r="F10" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A10&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G10" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A10&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H10" s="29">
         <f>IF(E10&gt;0,"À corriger",IF(D10+G10=B10,"Validée",IF(C10=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="29" t="inlineStr">
         <is>
           <t>27</t>
         </is>
       </c>
-      <c r="B11" s="11">
-        <f>COUNTIF(Tests!$C$5:$C$33,"*"&amp;A11&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C11" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A11&amp;"*",Tests!$F$5:$F$33,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D11" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A11&amp;"*",Tests!$G$5:$G$33,"OK")</f>
-        <v/>
-      </c>
-      <c r="E11" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A11&amp;"*",Tests!$G$5:$G$33,"KO")</f>
-        <v/>
-      </c>
-      <c r="F11" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A11&amp;"*",Tests!$G$5:$G$33,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G11" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A11&amp;"*",Tests!$G$5:$G$33,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H11" s="11">
+      <c r="B11" s="29">
+        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A11&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C11" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A11&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D11" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A11&amp;"*",Tests!$G$5:$G$41,"OK")</f>
+        <v/>
+      </c>
+      <c r="E11" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A11&amp;"*",Tests!$G$5:$G$41,"KO")</f>
+        <v/>
+      </c>
+      <c r="F11" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A11&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G11" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A11&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H11" s="29">
         <f>IF(E11&gt;0,"À corriger",IF(D11+G11=B11,"Validée",IF(C11=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="29" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="B12" s="11">
-        <f>COUNTIF(Tests!$C$5:$C$33,"*"&amp;A12&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C12" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A12&amp;"*",Tests!$F$5:$F$33,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D12" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A12&amp;"*",Tests!$G$5:$G$33,"OK")</f>
-        <v/>
-      </c>
-      <c r="E12" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A12&amp;"*",Tests!$G$5:$G$33,"KO")</f>
-        <v/>
-      </c>
-      <c r="F12" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A12&amp;"*",Tests!$G$5:$G$33,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G12" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A12&amp;"*",Tests!$G$5:$G$33,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H12" s="11">
+      <c r="B12" s="29">
+        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A12&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C12" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A12&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D12" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A12&amp;"*",Tests!$G$5:$G$41,"OK")</f>
+        <v/>
+      </c>
+      <c r="E12" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A12&amp;"*",Tests!$G$5:$G$41,"KO")</f>
+        <v/>
+      </c>
+      <c r="F12" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A12&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G12" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A12&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H12" s="29">
         <f>IF(E12&gt;0,"À corriger",IF(D12+G12=B12,"Validée",IF(C12=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="B13" s="11">
-        <f>COUNTIF(Tests!$C$5:$C$33,"*"&amp;A13&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C13" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A13&amp;"*",Tests!$F$5:$F$33,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D13" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A13&amp;"*",Tests!$G$5:$G$33,"OK")</f>
-        <v/>
-      </c>
-      <c r="E13" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A13&amp;"*",Tests!$G$5:$G$33,"KO")</f>
-        <v/>
-      </c>
-      <c r="F13" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A13&amp;"*",Tests!$G$5:$G$33,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G13" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A13&amp;"*",Tests!$G$5:$G$33,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H13" s="11">
+      <c r="B13" s="29">
+        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A13&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C13" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A13&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D13" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A13&amp;"*",Tests!$G$5:$G$41,"OK")</f>
+        <v/>
+      </c>
+      <c r="E13" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A13&amp;"*",Tests!$G$5:$G$41,"KO")</f>
+        <v/>
+      </c>
+      <c r="F13" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A13&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G13" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A13&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H13" s="29">
         <f>IF(E13&gt;0,"À corriger",IF(D13+G13=B13,"Validée",IF(C13=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="B14" s="11">
-        <f>COUNTIF(Tests!$C$5:$C$33,"*"&amp;A14&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C14" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A14&amp;"*",Tests!$F$5:$F$33,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D14" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A14&amp;"*",Tests!$G$5:$G$33,"OK")</f>
-        <v/>
-      </c>
-      <c r="E14" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A14&amp;"*",Tests!$G$5:$G$33,"KO")</f>
-        <v/>
-      </c>
-      <c r="F14" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A14&amp;"*",Tests!$G$5:$G$33,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G14" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A14&amp;"*",Tests!$G$5:$G$33,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H14" s="11">
+      <c r="B14" s="29">
+        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A14&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C14" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A14&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D14" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A14&amp;"*",Tests!$G$5:$G$41,"OK")</f>
+        <v/>
+      </c>
+      <c r="E14" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A14&amp;"*",Tests!$G$5:$G$41,"KO")</f>
+        <v/>
+      </c>
+      <c r="F14" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A14&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G14" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A14&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H14" s="29">
         <f>IF(E14&gt;0,"À corriger",IF(D14+G14=B14,"Validée",IF(C14=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="A15" s="29" t="inlineStr">
         <is>
           <t>31</t>
         </is>
       </c>
-      <c r="B15" s="11">
-        <f>COUNTIF(Tests!$C$5:$C$33,"*"&amp;A15&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C15" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A15&amp;"*",Tests!$F$5:$F$33,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D15" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A15&amp;"*",Tests!$G$5:$G$33,"OK")</f>
-        <v/>
-      </c>
-      <c r="E15" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A15&amp;"*",Tests!$G$5:$G$33,"KO")</f>
-        <v/>
-      </c>
-      <c r="F15" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A15&amp;"*",Tests!$G$5:$G$33,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G15" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A15&amp;"*",Tests!$G$5:$G$33,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H15" s="11">
+      <c r="B15" s="29">
+        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A15&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C15" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A15&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D15" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A15&amp;"*",Tests!$G$5:$G$41,"OK")</f>
+        <v/>
+      </c>
+      <c r="E15" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A15&amp;"*",Tests!$G$5:$G$41,"KO")</f>
+        <v/>
+      </c>
+      <c r="F15" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A15&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G15" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A15&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H15" s="29">
         <f>IF(E15&gt;0,"À corriger",IF(D15+G15=B15,"Validée",IF(C15=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="B16" s="11">
-        <f>COUNTIF(Tests!$C$5:$C$33,"*"&amp;A16&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C16" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A16&amp;"*",Tests!$F$5:$F$33,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D16" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A16&amp;"*",Tests!$G$5:$G$33,"OK")</f>
-        <v/>
-      </c>
-      <c r="E16" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A16&amp;"*",Tests!$G$5:$G$33,"KO")</f>
-        <v/>
-      </c>
-      <c r="F16" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A16&amp;"*",Tests!$G$5:$G$33,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G16" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A16&amp;"*",Tests!$G$5:$G$33,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H16" s="11">
+      <c r="B16" s="29">
+        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A16&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C16" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A16&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D16" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A16&amp;"*",Tests!$G$5:$G$41,"OK")</f>
+        <v/>
+      </c>
+      <c r="E16" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A16&amp;"*",Tests!$G$5:$G$41,"KO")</f>
+        <v/>
+      </c>
+      <c r="F16" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A16&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G16" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A16&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H16" s="29">
         <f>IF(E16&gt;0,"À corriger",IF(D16+G16=B16,"Validée",IF(C16=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="inlineStr">
+      <c r="A17" s="29" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="B17" s="11">
-        <f>COUNTIF(Tests!$C$5:$C$33,"*"&amp;A17&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C17" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A17&amp;"*",Tests!$F$5:$F$33,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D17" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A17&amp;"*",Tests!$G$5:$G$33,"OK")</f>
-        <v/>
-      </c>
-      <c r="E17" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A17&amp;"*",Tests!$G$5:$G$33,"KO")</f>
-        <v/>
-      </c>
-      <c r="F17" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A17&amp;"*",Tests!$G$5:$G$33,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G17" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A17&amp;"*",Tests!$G$5:$G$33,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H17" s="11">
+      <c r="B17" s="29">
+        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A17&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C17" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A17&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D17" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A17&amp;"*",Tests!$G$5:$G$41,"OK")</f>
+        <v/>
+      </c>
+      <c r="E17" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A17&amp;"*",Tests!$G$5:$G$41,"KO")</f>
+        <v/>
+      </c>
+      <c r="F17" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A17&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G17" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A17&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H17" s="29">
         <f>IF(E17&gt;0,"À corriger",IF(D17+G17=B17,"Validée",IF(C17=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="A18" s="29" t="inlineStr">
         <is>
           <t>34</t>
         </is>
       </c>
-      <c r="B18" s="11">
-        <f>COUNTIF(Tests!$C$5:$C$33,"*"&amp;A18&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C18" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A18&amp;"*",Tests!$F$5:$F$33,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D18" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A18&amp;"*",Tests!$G$5:$G$33,"OK")</f>
-        <v/>
-      </c>
-      <c r="E18" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A18&amp;"*",Tests!$G$5:$G$33,"KO")</f>
-        <v/>
-      </c>
-      <c r="F18" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A18&amp;"*",Tests!$G$5:$G$33,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G18" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A18&amp;"*",Tests!$G$5:$G$33,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H18" s="11">
+      <c r="B18" s="29">
+        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A18&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C18" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A18&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D18" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A18&amp;"*",Tests!$G$5:$G$41,"OK")</f>
+        <v/>
+      </c>
+      <c r="E18" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A18&amp;"*",Tests!$G$5:$G$41,"KO")</f>
+        <v/>
+      </c>
+      <c r="F18" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A18&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G18" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A18&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H18" s="29">
         <f>IF(E18&gt;0,"À corriger",IF(D18+G18=B18,"Validée",IF(C18=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="inlineStr">
+      <c r="A19" s="29" t="inlineStr">
         <is>
           <t>35</t>
         </is>
       </c>
-      <c r="B19" s="11">
-        <f>COUNTIF(Tests!$C$5:$C$33,"*"&amp;A19&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C19" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A19&amp;"*",Tests!$F$5:$F$33,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D19" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A19&amp;"*",Tests!$G$5:$G$33,"OK")</f>
-        <v/>
-      </c>
-      <c r="E19" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A19&amp;"*",Tests!$G$5:$G$33,"KO")</f>
-        <v/>
-      </c>
-      <c r="F19" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A19&amp;"*",Tests!$G$5:$G$33,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G19" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A19&amp;"*",Tests!$G$5:$G$33,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H19" s="11">
+      <c r="B19" s="29">
+        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A19&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C19" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A19&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D19" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A19&amp;"*",Tests!$G$5:$G$41,"OK")</f>
+        <v/>
+      </c>
+      <c r="E19" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A19&amp;"*",Tests!$G$5:$G$41,"KO")</f>
+        <v/>
+      </c>
+      <c r="F19" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A19&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G19" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A19&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H19" s="29">
         <f>IF(E19&gt;0,"À corriger",IF(D19+G19=B19,"Validée",IF(C19=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="inlineStr">
+      <c r="A20" s="29" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B20" s="11">
-        <f>COUNTIF(Tests!$C$5:$C$33,"*"&amp;A20&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C20" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A20&amp;"*",Tests!$F$5:$F$33,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D20" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A20&amp;"*",Tests!$G$5:$G$33,"OK")</f>
-        <v/>
-      </c>
-      <c r="E20" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A20&amp;"*",Tests!$G$5:$G$33,"KO")</f>
-        <v/>
-      </c>
-      <c r="F20" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A20&amp;"*",Tests!$G$5:$G$33,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G20" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A20&amp;"*",Tests!$G$5:$G$33,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H20" s="11">
+      <c r="B20" s="29">
+        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A20&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C20" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A20&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D20" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A20&amp;"*",Tests!$G$5:$G$41,"OK")</f>
+        <v/>
+      </c>
+      <c r="E20" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A20&amp;"*",Tests!$G$5:$G$41,"KO")</f>
+        <v/>
+      </c>
+      <c r="F20" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A20&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G20" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A20&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H20" s="29">
         <f>IF(E20&gt;0,"À corriger",IF(D20+G20=B20,"Validée",IF(C20=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="A21" s="29" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="B21" s="11">
-        <f>COUNTIF(Tests!$C$5:$C$33,"*"&amp;A21&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C21" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A21&amp;"*",Tests!$F$5:$F$33,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D21" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A21&amp;"*",Tests!$G$5:$G$33,"OK")</f>
-        <v/>
-      </c>
-      <c r="E21" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A21&amp;"*",Tests!$G$5:$G$33,"KO")</f>
-        <v/>
-      </c>
-      <c r="F21" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A21&amp;"*",Tests!$G$5:$G$33,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G21" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,"*"&amp;A21&amp;"*",Tests!$G$5:$G$33,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H21" s="11">
+      <c r="B21" s="29">
+        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A21&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C21" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A21&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D21" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A21&amp;"*",Tests!$G$5:$G$41,"OK")</f>
+        <v/>
+      </c>
+      <c r="E21" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A21&amp;"*",Tests!$G$5:$G$41,"KO")</f>
+        <v/>
+      </c>
+      <c r="F21" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A21&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G21" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A21&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H21" s="29">
         <f>IF(E21&gt;0,"À corriger",IF(D21+G21=B21,"Validée",IF(C21=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="inlineStr">
+      <c r="A22" s="29" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B22" s="29">
+        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A22&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C22" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A22&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D22" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A22&amp;"*",Tests!$G$5:$G$41,"OK")</f>
+        <v/>
+      </c>
+      <c r="E22" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A22&amp;"*",Tests!$G$5:$G$41,"KO")</f>
+        <v/>
+      </c>
+      <c r="F22" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A22&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G22" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A22&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H22" s="29">
+        <f>IF(E22&gt;0,"À corriger",IF(D22+G22=B22,"Validée",IF(C22=0,"À tester","En cours")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="29" t="inlineStr">
         <is>
           <t>5 (en attente)</t>
         </is>
       </c>
-      <c r="B22" s="11">
-        <f>COUNTIF(Tests!$C$5:$C$33,A22)</f>
-        <v/>
-      </c>
-      <c r="C22" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,A22,Tests!$F$5:$F$33,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D22" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,A22,Tests!$G$5:$G$33,"OK")</f>
-        <v/>
-      </c>
-      <c r="E22" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,A22,Tests!$G$5:$G$33,"KO")</f>
-        <v/>
-      </c>
-      <c r="F22" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,A22,Tests!$G$5:$G$33,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G22" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,A22,Tests!$G$5:$G$33,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H22" s="11">
-        <f>IF(E22&gt;0,"À corriger",IF(D22+G22=B22,"Validée",IF(C22=0,"À tester","En cours")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="11" t="inlineStr">
+      <c r="B23" s="29">
+        <f>COUNTIF(Tests!$C$5:$C$41,A23)</f>
+        <v/>
+      </c>
+      <c r="C23" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,A23,Tests!$F$5:$F$41,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D23" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,A23,Tests!$G$5:$G$41,"OK")</f>
+        <v/>
+      </c>
+      <c r="E23" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,A23,Tests!$G$5:$G$41,"KO")</f>
+        <v/>
+      </c>
+      <c r="F23" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,A23,Tests!$G$5:$G$41,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G23" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,A23,Tests!$G$5:$G$41,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H23" s="29">
+        <f>IF(E23&gt;0,"À corriger",IF(D23+G23=B23,"Validée",IF(C23=0,"À tester","En cours")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="29" t="inlineStr">
         <is>
           <t>SYNC</t>
         </is>
       </c>
-      <c r="B23" s="11">
-        <f>COUNTIF(Tests!$C$5:$C$33,A23)</f>
-        <v/>
-      </c>
-      <c r="C23" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,A23,Tests!$F$5:$F$33,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D23" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,A23,Tests!$G$5:$G$33,"OK")</f>
-        <v/>
-      </c>
-      <c r="E23" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,A23,Tests!$G$5:$G$33,"KO")</f>
-        <v/>
-      </c>
-      <c r="F23" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,A23,Tests!$G$5:$G$33,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G23" s="11">
-        <f>COUNTIFS(Tests!$C$5:$C$33,A23,Tests!$G$5:$G$33,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H23" s="11">
-        <f>IF(E23&gt;0,"À corriger",IF(D23+G23=B23,"Validée",IF(C23=0,"À tester","En cours")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="12" t="inlineStr">
+      <c r="B24" s="29">
+        <f>COUNTIF(Tests!$C$5:$C$41,A24)</f>
+        <v/>
+      </c>
+      <c r="C24" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,A24,Tests!$F$5:$F$41,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D24" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,A24,Tests!$G$5:$G$41,"OK")</f>
+        <v/>
+      </c>
+      <c r="E24" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,A24,Tests!$G$5:$G$41,"KO")</f>
+        <v/>
+      </c>
+      <c r="F24" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,A24,Tests!$G$5:$G$41,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G24" s="29">
+        <f>COUNTIFS(Tests!$C$5:$C$41,A24,Tests!$G$5:$G$41,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H24" s="29">
+        <f>IF(E24&gt;0,"À corriger",IF(D24+G24=B24,"Validée",IF(C24=0,"À tester","En cours")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="30" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B24" s="12">
-        <f>COUNTA(Tests!$A$5:$A$33)</f>
-        <v/>
-      </c>
-      <c r="C24" s="12">
-        <f>COUNTIF(Tests!$F$5:$F$33,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D24" s="12">
-        <f>COUNTIF(Tests!$G$5:$G$33,"OK")</f>
-        <v/>
-      </c>
-      <c r="E24" s="12">
-        <f>COUNTIF(Tests!$G$5:$G$33,"KO")</f>
-        <v/>
-      </c>
-      <c r="F24" s="12">
-        <f>COUNTIF(Tests!$G$5:$G$33,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G24" s="12">
-        <f>COUNTIF(Tests!$G$5:$G$33,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H24" s="12" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="13" t="inlineStr">
-        <is>
-          <t>Un test peut couvrir plusieurs PR (ex. test 11) : il compte pour chacune. « Validée » = tous les tests de la PR en OK ou Non testable.</t>
-        </is>
-      </c>
+      <c r="B25" s="30">
+        <f>COUNTA(Tests!$A$5:$A$41)</f>
+        <v/>
+      </c>
+      <c r="C25" s="30">
+        <f>COUNTIF(Tests!$F$5:$F$41,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D25" s="30">
+        <f>COUNTIF(Tests!$G$5:$G$41,"OK")</f>
+        <v/>
+      </c>
+      <c r="E25" s="30">
+        <f>COUNTIF(Tests!$G$5:$G$41,"KO")</f>
+        <v/>
+      </c>
+      <c r="F25" s="30">
+        <f>COUNTIF(Tests!$G$5:$G$41,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G25" s="30">
+        <f>COUNTIF(Tests!$G$5:$G$41,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H25" s="30" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="inlineStr">
-        <is>
-          <t>« 5 (en attente) » : test resté en stand-by de la PR 5 (fusionnée). « SYNC » : analyse de départ, sans PR propre.</t>
+      <c r="A27" s="31" t="inlineStr">
+        <is>
+          <t>Un test peut couvrir plusieurs PR : il compte pour chacune. « Validée » = tous les tests de la PR en OK ou Non testable. Un test « Partiel » corrigé depuis reste « En cours » jusqu'à ce que tu le refasses.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H4:H23">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="1">
+  <conditionalFormatting sqref="H4:H24">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="6">
       <formula>"Validée"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="7">
       <formula>"À corriger"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2784,7 +3397,7 @@
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>https://github.com/Herve-obe/VERIFLOW-v4/actions/runs/39635810261 (artefact veriflow-windows-latest).</t>
+          <t>https://github.com/Herve-obe/VERIFLOW-v4/actions/runs/40104706786 (artefact veriflow-windows-latest, build du 24/10).</t>
         </is>
       </c>
     </row>
@@ -2800,6 +3413,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="16.5" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Recette : retours du 26/10 et nouveaux tests 38 et 39
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MoqekrFvgrWkuAe5NHnE5A
</commit_message>
<xml_diff>
--- a/docs/recette/RECETTE_PR_17-37.xlsx
+++ b/docs/recette/RECETTE_PR_17-37.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Légende" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tests'!$A$4:$J$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tests'!$A$4:$J$43</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Tests'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -23,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,17 +60,6 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="FF595959"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
       <sz val="10"/>
     </font>
     <font>
@@ -87,20 +76,22 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="00595959"/>
+      <color rgb="FF595959"/>
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -119,7 +110,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD9E1F2"/>
+        <fgColor rgb="FF1F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -129,7 +135,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE2EFDA"/>
+        <fgColor rgb="FFD9E1F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -142,23 +148,28 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -209,7 +220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -232,34 +243,24 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -268,28 +269,49 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="14" fontId="4" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="11" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -723,11 +745,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -801,13 +823,13 @@
           <t>Commentaires</t>
         </is>
       </c>
-      <c r="J4" s="18" t="inlineStr">
-        <is>
-          <t>Réponse de Claude (mise à jour 25/10)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="25.5" customHeight="1">
+      <c r="J4" s="14" t="inlineStr">
+        <is>
+          <t>Réponse de Claude (mise à jour 27/10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" hidden="1" ht="25.5" customHeight="1">
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
@@ -849,9 +871,9 @@
           <t>RAS</t>
         </is>
       </c>
-      <c r="J5" s="19" t="n"/>
-    </row>
-    <row r="6" ht="25.5" customHeight="1">
+      <c r="J5" s="15" t="n"/>
+    </row>
+    <row r="6" hidden="1" ht="25.5" customHeight="1">
       <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
@@ -893,9 +915,9 @@
           <t>RAS</t>
         </is>
       </c>
-      <c r="J6" s="19" t="n"/>
-    </row>
-    <row r="7" ht="25.5" customHeight="1">
+      <c r="J6" s="15" t="n"/>
+    </row>
+    <row r="7" hidden="1" ht="25.5" customHeight="1">
       <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
@@ -937,9 +959,9 @@
           <t>RAS</t>
         </is>
       </c>
-      <c r="J7" s="19" t="n"/>
-    </row>
-    <row r="8" ht="25.5" customHeight="1">
+      <c r="J7" s="15" t="n"/>
+    </row>
+    <row r="8" ht="89.25" customHeight="1">
       <c r="A8" s="4" t="n">
         <v>4</v>
       </c>
@@ -974,20 +996,20 @@
         </is>
       </c>
       <c r="H8" s="7" t="n">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>Ajouter des images du logiciel avec mise en avant des points mentionnés</t>
-        </is>
-      </c>
-      <c r="J8" s="21" t="inlineStr">
-        <is>
-          <t>Captures du guide avec les points mis en évidence : à faire (PR à venir).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="25.5" customHeight="1">
+          <t>Ajouter des images du logiciel avec mise en avant des points mentionnés dans la version html dispo dans le logiciel + au lancement de Veriflow, l'application s'ouvre à chaque en mode fenêtre, il faut qu'elle s'ouvre par défaut fenêtre ajustée à la taille de l'écran et retienne le réglage si l'utilisateur laisse ainsi et ferme ou s'il l'a laissé en mode fenêtre.</t>
+        </is>
+      </c>
+      <c r="J8" s="28" t="inlineStr">
+        <is>
+          <t>Fenêtre agrandie au premier lancement, taille et état retenus : fait, voir test 39 (build du 27/10 (run 40517638115)). Captures dans le guide : à faire (PR à venir).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" hidden="1" ht="25.5" customHeight="1">
       <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
@@ -1029,9 +1051,9 @@
           <t>RAS</t>
         </is>
       </c>
-      <c r="J9" s="19" t="n"/>
-    </row>
-    <row r="10" ht="63.75" customHeight="1">
+      <c r="J9" s="15" t="n"/>
+    </row>
+    <row r="10" hidden="1" ht="63.75" customHeight="1">
       <c r="A10" s="4" t="n">
         <v>6</v>
       </c>
@@ -1073,13 +1095,13 @@
           <t>RAS</t>
         </is>
       </c>
-      <c r="J10" s="20" t="inlineStr">
+      <c r="J10" s="16" t="inlineStr">
         <is>
           <t>Corrigé : bouton « Valider » (applique tout de suite aux onglets et lecteurs ouverts), « Annuler », « Valeurs d'usine » par rubrique. « Remettre à zéro maintenant » renommé « Vider l'état de travail » : il vide les destinations et dossiers en cours, pas les Préférences. À refaire dans le nouveau build.</t>
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" hidden="1">
       <c r="A11" s="4" t="n">
         <v>7</v>
       </c>
@@ -1121,9 +1143,9 @@
           <t>RAS</t>
         </is>
       </c>
-      <c r="J11" s="19" t="n"/>
-    </row>
-    <row r="12" ht="25.5" customHeight="1">
+      <c r="J11" s="15" t="n"/>
+    </row>
+    <row r="12" hidden="1" ht="25.5" customHeight="1">
       <c r="A12" s="4" t="n">
         <v>8</v>
       </c>
@@ -1165,9 +1187,9 @@
           <t>RAS</t>
         </is>
       </c>
-      <c r="J12" s="19" t="n"/>
-    </row>
-    <row r="13" ht="25.5" customHeight="1">
+      <c r="J12" s="15" t="n"/>
+    </row>
+    <row r="13" hidden="1" ht="25.5" customHeight="1">
       <c r="A13" s="4" t="n">
         <v>9</v>
       </c>
@@ -1209,9 +1231,9 @@
           <t>RAS</t>
         </is>
       </c>
-      <c r="J13" s="19" t="n"/>
-    </row>
-    <row r="14" ht="38.25" customHeight="1">
+      <c r="J13" s="15" t="n"/>
+    </row>
+    <row r="14" hidden="1" ht="38.25" customHeight="1">
       <c r="A14" s="4" t="n">
         <v>10</v>
       </c>
@@ -1253,13 +1275,13 @@
           <t>RAS</t>
         </is>
       </c>
-      <c r="J14" s="20" t="inlineStr">
+      <c r="J14" s="16" t="inlineStr">
         <is>
           <t>Test reformulé (colonne Action) : il vérifie que VERIFLOW reconnaît le type de carte d'après ses dossiers. Sans carte caméra, ou sans dossier qui a gardé la structure d'origine, marque « Non testable » et vérifie seulement l'aperçu du chemin.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="38.25" customHeight="1">
+    <row r="15" hidden="1" ht="38.25" customHeight="1">
       <c r="A15" s="4" t="n">
         <v>11</v>
       </c>
@@ -1301,13 +1323,13 @@
           <t>Dans l'explorer de Veriflow, il y a un icone "ejecter" à côté des disques externes, cartes…etc, il faudrait que cet icône permette aussi d'éjecter ces supports en toute sécurité</t>
         </is>
       </c>
-      <c r="J15" s="21" t="inlineStr">
+      <c r="J15" s="17" t="inlineStr">
         <is>
           <t>Bouton ⏏ de l'explorateur : fait, voir test 30 (build du 24/10 (run 40104706786)).</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="25.5" customHeight="1">
+    <row r="16" hidden="1" ht="25.5" customHeight="1">
       <c r="A16" s="4" t="n">
         <v>12</v>
       </c>
@@ -1349,9 +1371,9 @@
           <t>RAS</t>
         </is>
       </c>
-      <c r="J16" s="19" t="n"/>
-    </row>
-    <row r="17" ht="25.5" customHeight="1">
+      <c r="J16" s="15" t="n"/>
+    </row>
+    <row r="17" hidden="1" ht="25.5" customHeight="1">
       <c r="A17" s="4" t="n">
         <v>13</v>
       </c>
@@ -1393,13 +1415,13 @@
           <t>RAS</t>
         </is>
       </c>
-      <c r="J17" s="20" t="inlineStr">
+      <c r="J17" s="16" t="inlineStr">
         <is>
           <t>À refaire après le test 11.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="63.75" customHeight="1">
+    <row r="18" hidden="1" ht="63.75" customHeight="1">
       <c r="A18" s="4" t="n">
         <v>14</v>
       </c>
@@ -1430,24 +1452,24 @@
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>Partiel</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
-        <v>46319</v>
+        <v>46321</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
           <t>Fenêtre glissée sur le 2e écran, double clic dans la barre du haut pour adapter à la taille de l'écran (pas en plein écran, juste fenêtre adaptée). Echap, ferme le lecteur pop-up. Double clic sur le même rush, le lecteur pop-up se rouvre sur le 1er écran, pas sur le 2e</t>
         </is>
       </c>
-      <c r="J18" s="21" t="inlineStr">
+      <c r="J18" s="17" t="inlineStr">
         <is>
           <t>Corrigé : place mémorisée en pixels réels et fenêtre agrandie rétablie sur le même écran. À refaire avec le build du 24/10 (run 40104706786).</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="25.5" customHeight="1">
+    <row r="19" hidden="1" ht="25.5" customHeight="1">
       <c r="A19" s="4" t="n">
         <v>15</v>
       </c>
@@ -1489,7 +1511,7 @@
           <t>Même protocole, pas en plein écran, juste fenêtre adaptée, la fenêtre reste bien en place et lance le 2e rush</t>
         </is>
       </c>
-      <c r="J19" s="19" t="n"/>
+      <c r="J19" s="15" t="n"/>
     </row>
     <row r="20" ht="63.75" customHeight="1">
       <c r="A20" s="4" t="n">
@@ -1526,16 +1548,16 @@
         </is>
       </c>
       <c r="H20" s="7" t="n">
-        <v>46319</v>
+        <v>46321</v>
       </c>
       <c r="I20" s="8" t="inlineStr">
         <is>
-          <t>Lecteur pop-up déplacé sur le 2e écran, sortie TV choisie, affichage plein écran. Curseur souris disparait au bout de 2 sec et réapparait si je le bouge, mais de contrôle de lecture possible avec espace : le contrôle est resté sur le choix du moniteur !</t>
-        </is>
-      </c>
-      <c r="J20" s="21" t="inlineStr">
-        <is>
-          <t>Corrigé : après le choix du moniteur, le clavier revient au lecteur (Espace, J/K/L). À refaire avec le build du 24/10 (run 40104706786).</t>
+          <t>Lecteur pop-up déplacé sur le 2e écran, sortie TV choisie, affichage plein écran. Curseur souris disparait au bout de 2 sec et réapparait si je le bouge, mais pas de contrôle de lecture possible avec espace : ne fonctionne que quand le lecteur n'est pas en plein écran.</t>
+        </is>
+      </c>
+      <c r="J20" s="28" t="inlineStr">
+        <is>
+          <t>Corrigé : après l'ouverture du moniteur, le clavier revient au lecteur (un clic sur le moniteur le lui donne, Échap le ferme). À refaire avec le build du 27/10 (run 40517638115).</t>
         </is>
       </c>
     </row>
@@ -1574,16 +1596,16 @@
         </is>
       </c>
       <c r="H21" s="7" t="n">
-        <v>46319</v>
+        <v>46321</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
           <t>Lecteur pop-up ouvert sur le 2e écran. Je débranche le 2e écran, le lecteur revient sur l'écran principal. Je ferme le lecteur pop-up, je double clic sur un rush, le lecteur pop-up s'ouvre sur l'écran principal (toujours pas de 2e écran branché) mais message d'erreur audio (voir capture)</t>
         </is>
       </c>
-      <c r="J21" s="21" t="inlineStr">
-        <is>
-          <t>Corrigé : la carte son est ouverte sur un fil neuf (erreur « mode thread » de Windows). À refaire avec le build du 24/10 (run 40104706786).</t>
+      <c r="J21" s="28" t="inlineStr">
+        <is>
+          <t>Cause trouvée : la sortie « par défaut du système » de Windows refuse le mode COM choisi par la bibliothèque audio. Les fils audio passent en mode multithread avant elle. À refaire avec le build du 27/10 (run 40517638115).</t>
         </is>
       </c>
     </row>
@@ -1622,17 +1644,17 @@
         </is>
       </c>
       <c r="H22" s="7" t="n">
-        <v>46319</v>
+        <v>46321</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
-          <t>Test sur média plus petit, player pop-up, le son arrive au bout de quelques secondes après le début de lecture.
-Metadata : l'enregistrement des modif ne se fait que par un clic sur le bouton enregistrer, il faut ajouter la validation par la touche Return et la touche entrée du pavé numérique du clavier + bouton enregistrer superposé à la colonne de manière non esthétique. Dans la fenêtre centrale, le TC n'est pas affiché. (voir capture) + impossible de redimenssioner les colonnes à la main ni changer qeulle colonne sont visible/invisible</t>
-        </is>
-      </c>
-      <c r="J22" s="21" t="inlineStr">
-        <is>
-          <t>Corrigé : Entrée (clavier et pavé numérique), barre Enregistrer, TC des WAV : voir test 34. Son en retard : à revérifier avec le build du 24/10 (run 40104706786) (peut venir de l'erreur audio du test 17). Colonnes réglables et masquables : à faire (PR à venir).</t>
+          <t xml:space="preserve">Double clic sur un media audio ouvre le player pop-up mais demande de charger un media (voir capture).
+</t>
+        </is>
+      </c>
+      <c r="J22" s="28" t="inlineStr">
+        <is>
+          <t>Même cause que le test 17 : le son ne s'ouvrait pas, et la vue restait vide. L'erreur éventuelle s'affiche maintenant dans la vue. À refaire avec le build du 27/10 (run 40517638115).</t>
         </is>
       </c>
     </row>
@@ -1668,7 +1690,7 @@
       <c r="G23" s="6" t="n"/>
       <c r="H23" s="7" t="n"/>
       <c r="I23" s="8" t="n"/>
-      <c r="J23" s="19" t="n"/>
+      <c r="J23" s="15" t="n"/>
     </row>
     <row r="24" ht="153" customHeight="1">
       <c r="A24" s="4" t="n">
@@ -1701,26 +1723,25 @@
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>Partiel</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
-        <v>46319</v>
+        <v>46321</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
-          <t>Création d'un projet, nom du projet pas centré sur le haut de la fenêtre. Case cochée dans les préférences. Je n'ai pas compris la suite du protocole. Explique moi pas à pas.
-J'ai essayé d'ouvrir plusieurs rushes audio dans l'onglet PLAYER : ils sont tous ouverts en même temps et l'affichage de l'application s'est décalé. Pour pouvoir lire plusieurs rushes dans PLAYER, il faut créer un système de liste de lecture.
-Dans les consles audio du PLAYER, le clic sur les boutons SOLO et/ou MUTE ne fais que noircir le bouton, il faut qu'il passe en couleur pour le mettre en évidence.</t>
-        </is>
-      </c>
-      <c r="J24" s="21" t="inlineStr">
-        <is>
-          <t>Test réécrit pas à pas (colonne Action). Projet centré et SOLO/MUTE : voir tests 32 et 33. Liste de lecture du PLAYER : à faire (PR à venir).</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="25.5" customHeight="1">
+          <t>Fonctionnel mais je ne comprends pas l'utilité.
+Il serait plus intéressant de pouvoir avoir accès aussi à l'explorer sur la gauche de l'application comme dans OFFLOAD et MEDIA.</t>
+        </is>
+      </c>
+      <c r="J24" s="28" t="inlineStr">
+        <is>
+          <t>Utilité : en visionnant les prises une à une, la ligne du rapport s'ouvre seule, sans appuyer sur R. Explorateur à gauche dans le PLAYER : noté, à faire avec la liste de lecture (PR à venir).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" hidden="1" ht="25.5" customHeight="1">
       <c r="A25" s="4" t="n">
         <v>21</v>
       </c>
@@ -1762,7 +1783,7 @@
           <t>RAS</t>
         </is>
       </c>
-      <c r="J25" s="19" t="n"/>
+      <c r="J25" s="15" t="n"/>
     </row>
     <row r="26" ht="25.5" customHeight="1">
       <c r="A26" s="4" t="n">
@@ -1796,9 +1817,9 @@
       <c r="G26" s="6" t="n"/>
       <c r="H26" s="7" t="n"/>
       <c r="I26" s="8" t="n"/>
-      <c r="J26" s="19" t="n"/>
-    </row>
-    <row r="27">
+      <c r="J26" s="15" t="n"/>
+    </row>
+    <row r="27" ht="89.25" customHeight="1">
       <c r="A27" s="4" t="n">
         <v>23</v>
       </c>
@@ -1824,13 +1845,27 @@
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="n"/>
-      <c r="H27" s="7" t="n"/>
-      <c r="I27" s="8" t="n"/>
-      <c r="J27" s="19" t="n"/>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="n">
+        <v>46321</v>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>Si j'ai bien compris : j'ai importé plusieurs rushes vidéo et plusieurs audio dans l'onglet SYNC, quand je déplace la souris sur une colonne et j'utilise la molette, seule la colonne que je survole défile (Explorer, Vidéo ou Audio). Par contre, j'ai remarqué que "Vidéo" et "Audio" sont écrit tout à gauche, il faudrait que chacun soit au dessus de sa colonne (voir capture)</t>
+        </is>
+      </c>
+      <c r="J27" s="28" t="inlineStr">
+        <is>
+          <t>Oui, c'est le bon protocole : test OK pour le défilement. Titres « Vidéos » et « Sons » au-dessus de chaque liste : fait. À revoir avec le build du 27/10 (run 40517638115).</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="51" customHeight="1">
       <c r="A28" s="4" t="n">
@@ -1863,24 +1898,24 @@
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>Partiel</t>
+          <t>KO</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
-        <v>46319</v>
+        <v>46321</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
-          <t>Mode AUDIO : pas de choix du dossier pour les fichier resynchro - direct dans le dossier des rushes vidéo. Fichiers resynchro ouvert dans Resolve : que de l'audio, pas de vidéo.</t>
-        </is>
-      </c>
-      <c r="J28" s="21" t="inlineStr">
-        <is>
-          <t>Image absente dans Resolve : limite de Resolve gratuit (H.264 10 bits 4:2:2), lu dans Premiere. Mauvais son : corrigé, voir tests 35 à 37. Choix du dossier en mode AUDIO : envoie-moi une capture de la colonne de droite si le problème revient.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
+          <t>Il manque des réglages dans la partie droite (voir captures)</t>
+        </is>
+      </c>
+      <c r="J28" s="28" t="inlineStr">
+        <is>
+          <t>Corrigé : la destination et les options d'export sont visibles dès le départ (bouton actif après l'analyse). À refaire avec le build du 27/10 (run 40517638115).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" hidden="1">
       <c r="A29" s="4" t="n">
         <v>25</v>
       </c>
@@ -1922,9 +1957,9 @@
           <t>RAS</t>
         </is>
       </c>
-      <c r="J29" s="19" t="n"/>
-    </row>
-    <row r="30" ht="38.25" customHeight="1">
+      <c r="J29" s="15" t="n"/>
+    </row>
+    <row r="30" hidden="1" ht="63.75" customHeight="1">
       <c r="A30" s="4" t="n">
         <v>26</v>
       </c>
@@ -1950,23 +1985,29 @@
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G30" s="6" t="n"/>
-      <c r="H30" s="7" t="n"/>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="n">
+        <v>46321</v>
+      </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
-          <t>Je ne comprends pas, explique pas à pas</t>
-        </is>
-      </c>
-      <c r="J30" s="21" t="inlineStr">
+          <t>RAS</t>
+        </is>
+      </c>
+      <c r="J30" s="17" t="inlineStr">
         <is>
           <t>Test réécrit pas à pas (colonne Action).</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="38.25" customHeight="1">
+    <row r="31" hidden="1" ht="38.25" customHeight="1">
       <c r="A31" s="4" t="n">
         <v>27</v>
       </c>
@@ -1992,23 +2033,29 @@
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="n"/>
-      <c r="H31" s="7" t="n"/>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="n">
+        <v>46321</v>
+      </c>
       <c r="I31" s="8" t="inlineStr">
         <is>
-          <t>Je ne comprends pas, explique pas à pas</t>
-        </is>
-      </c>
-      <c r="J31" s="21" t="inlineStr">
+          <t>RAS</t>
+        </is>
+      </c>
+      <c r="J31" s="17" t="inlineStr">
         <is>
           <t>Test réécrit pas à pas (colonne Action).</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="25.5" customHeight="1">
+    <row r="32" hidden="1" ht="25.5" customHeight="1">
       <c r="A32" s="4" t="n">
         <v>28</v>
       </c>
@@ -2039,24 +2086,24 @@
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>Non testable</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
-        <v>46319</v>
+        <v>46321</v>
       </c>
       <c r="I32" s="8" t="inlineStr">
         <is>
-          <t>Il n'y a plus l'option "repartir de zéro", seulement "vider l'état de travail" ou "Effacer toutes les données"</t>
-        </is>
-      </c>
-      <c r="J32" s="21" t="inlineStr">
+          <t>Garder tout de même le réglage par défaut de l'applicaiton qui s'ouvre en grande fenêtre ajustée à l'écran. (voir test 4)</t>
+        </is>
+      </c>
+      <c r="J32" s="17" t="inlineStr">
         <is>
           <t>L'option est dans la liste déroulante « À l'ouverture de VERIFLOW » (Préférences &gt; Général), au-dessus des deux boutons. À refaire.</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="38.25" customHeight="1">
+    <row r="33" hidden="1" ht="38.25" customHeight="1">
       <c r="A33" s="4" t="n">
         <v>29</v>
       </c>
@@ -2087,330 +2134,464 @@
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="n">
+        <v>46321</v>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>RAS</t>
+        </is>
+      </c>
+      <c r="J33" s="17" t="inlineStr">
+        <is>
+          <t>Corrigé : installation dans C:\Program Files\VERIFLOW (droits administrateur demandés). Désinstalle d'abord l'ancienne version (AppData). À refaire avec le build du 24/10 (run 40104706786).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="38.25" customHeight="1">
+      <c r="A34" s="18" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="19" t="inlineStr">
+        <is>
+          <t>B. OFFLOAD</t>
+        </is>
+      </c>
+      <c r="C34" s="18" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D34" s="19" t="inlineStr">
+        <is>
+          <t>Explorateur : cliquer sur le bouton ⏏ à côté d'un disque externe ou d'une carte.</t>
+        </is>
+      </c>
+      <c r="E34" s="19" t="inlineStr">
+        <is>
+          <t>Barre d'état : « Éjecté, tu peux le débrancher ». Le disque disparaît de l'explorateur. En cas de refus, le message donne la raison de Windows.</t>
+        </is>
+      </c>
+      <c r="F34" s="20" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G34" s="20" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="H34" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="I34" s="22" t="inlineStr">
+        <is>
+          <t>ejection impossible (voir capture)</t>
+        </is>
+      </c>
+      <c r="J34" s="28" t="inlineStr">
+        <is>
+          <t>La capture de l'éjection n'est pas arrivée (5 captures reçues : SYNC, lecteur rapide). Recopie le message de la barre d'état en bas ici, ou renvoie la capture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" hidden="1">
+      <c r="A35" s="18" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="19" t="inlineStr">
+        <is>
+          <t>B. OFFLOAD</t>
+        </is>
+      </c>
+      <c r="C35" s="18" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D35" s="19" t="inlineStr">
+        <is>
+          <t>Explorateur : déplier le disque HERVE EDU (F:).</t>
+        </is>
+      </c>
+      <c r="E35" s="19" t="inlineStr">
+        <is>
+          <t>Les dossiers FOUND.000 à FOUND.004 n'apparaissent plus.</t>
+        </is>
+      </c>
+      <c r="F35" s="20" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G35" s="20" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H35" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="I35" s="22" t="inlineStr">
+        <is>
+          <t>RAS</t>
+        </is>
+      </c>
+      <c r="J35" s="23" t="inlineStr">
+        <is>
+          <t>Nouveau test (correctifs du 24/10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="63.75" customHeight="1">
+      <c r="A36" s="18" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="19" t="inlineStr">
+        <is>
+          <t>D. PLAYER</t>
+        </is>
+      </c>
+      <c r="C36" s="18" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="D36" s="19" t="inlineStr">
+        <is>
+          <t>PLAYER en mode AUDIO : cliquer SOLO puis MUTE sur une piste.</t>
+        </is>
+      </c>
+      <c r="E36" s="19" t="inlineStr">
+        <is>
+          <t>SOLO en orange, MUTE en rouge quand ils sont actifs.</t>
+        </is>
+      </c>
+      <c r="F36" s="20" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G36" s="20" t="inlineStr">
+        <is>
           <t>Partiel</t>
         </is>
       </c>
-      <c r="H33" s="7" t="n">
-        <v>46319</v>
-      </c>
-      <c r="I33" s="8" t="inlineStr">
-        <is>
-          <t>Il faut que l'install se fasse dans le dossier Programme et non dans le dossier AppData (voir capture). Sinon, logiciel bien réintsallé à zéro.</t>
-        </is>
-      </c>
-      <c r="J33" s="21" t="inlineStr">
-        <is>
-          <t>Corrigé : installation dans C:\Program Files\VERIFLOW (droits administrateur demandés). Désinstalle d'abord l'ancienne version (AppData). À refaire avec le build du 24/10 (run 40104706786).</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="22" t="n">
-        <v>30</v>
-      </c>
-      <c r="B34" s="23" t="inlineStr">
-        <is>
-          <t>B. OFFLOAD</t>
-        </is>
-      </c>
-      <c r="C34" s="22" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="D34" s="23" t="inlineStr">
-        <is>
-          <t>Explorateur : cliquer sur le bouton ⏏ à côté d'un disque externe ou d'une carte.</t>
-        </is>
-      </c>
-      <c r="E34" s="23" t="inlineStr">
-        <is>
-          <t>Barre d'état : « Éjecté, tu peux le débrancher ». Le disque disparaît de l'explorateur. En cas de refus, le message donne la raison de Windows.</t>
-        </is>
-      </c>
-      <c r="F34" s="24" t="inlineStr">
+      <c r="H36" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="I36" s="22" t="inlineStr">
+        <is>
+          <t>Ok pour les mise en couleur mais : le bouton MUTE doit être prioritaire sur le bouton SOLO, si une piste est en MUTE et en SOLO, alors elle est MUTE.
+Il faut aussi ajouter un bouton SOLO pour chaque piste de la console du mode VIDEO.</t>
+        </is>
+      </c>
+      <c r="J36" s="28" t="inlineStr">
+        <is>
+          <t>Corrigé : MUTE prime sur SOLO ; bouton S ajouté sur chaque piste en mode VIDEO. Voir test 38 (build du 27/10 (run 40517638115)).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="18" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="19" t="inlineStr">
+        <is>
+          <t>A. Installation et menus</t>
+        </is>
+      </c>
+      <c r="C37" s="18" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="D37" s="19" t="inlineStr">
+        <is>
+          <t>Ouvrir un projet et regarder la barre du haut.</t>
+        </is>
+      </c>
+      <c r="E37" s="19" t="inlineStr">
+        <is>
+          <t>Nom du projet au centre de la fenêtre.</t>
+        </is>
+      </c>
+      <c r="F37" s="20" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G37" s="20" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H37" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="I37" s="22" t="inlineStr">
+        <is>
+          <t>RAS</t>
+        </is>
+      </c>
+      <c r="J37" s="23" t="inlineStr">
+        <is>
+          <t>Nouveau test (correctifs du 24/10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="38.25" customHeight="1">
+      <c r="A38" s="18" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="19" t="inlineStr">
+        <is>
+          <t>C. MEDIA et second écran</t>
+        </is>
+      </c>
+      <c r="C38" s="18" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="D38" s="19" t="inlineStr">
+        <is>
+          <t>MEDIA : modifier un champ, puis Entrée (clavier principal), puis un autre avec Entrée du pavé numérique. Regarder la barre Enregistrer et la colonne TC en mode AUDIO.</t>
+        </is>
+      </c>
+      <c r="E38" s="19" t="inlineStr">
+        <is>
+          <t>Enregistré à chaque Entrée ; barre Enregistrer sur toute la largeur, séparée des champs ; TC affiché pour les WAV.</t>
+        </is>
+      </c>
+      <c r="F38" s="20" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="G38" s="20" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H38" s="21" t="n">
+        <v>46321</v>
+      </c>
+      <c r="I38" s="22" t="inlineStr">
+        <is>
+          <t>RAS</t>
+        </is>
+      </c>
+      <c r="J38" s="23" t="inlineStr">
+        <is>
+          <t>Nouveau test (correctifs du 24/10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="25.5" customHeight="1">
+      <c r="A39" s="18" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="19" t="inlineStr">
+        <is>
+          <t>E. SYNC</t>
+        </is>
+      </c>
+      <c r="C39" s="18" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="D39" s="19" t="inlineStr">
+        <is>
+          <t>SYNC : un rush vidéo avec LTC sur une piste et son témoin sur l'autre, avec son WAV. Méthode Automatique, Analyser.</t>
+        </is>
+      </c>
+      <c r="E39" s="19" t="inlineStr">
+        <is>
+          <t>Colonne Méthode : LTC ; badge LTC à côté du timecode ; TC = celui du LTC (pas l'horloge de la Panasonic).</t>
+        </is>
+      </c>
+      <c r="F39" s="20" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="G34" s="24" t="inlineStr"/>
-      <c r="H34" s="25" t="n"/>
-      <c r="I34" s="26" t="inlineStr"/>
-      <c r="J34" s="27" t="inlineStr">
+      <c r="G39" s="20" t="n"/>
+      <c r="H39" s="21" t="n"/>
+      <c r="I39" s="22" t="n"/>
+      <c r="J39" s="23" t="inlineStr">
         <is>
           <t>Nouveau test (correctifs du 24/10).</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="22" t="n">
-        <v>31</v>
-      </c>
-      <c r="B35" s="23" t="inlineStr">
-        <is>
-          <t>B. OFFLOAD</t>
-        </is>
-      </c>
-      <c r="C35" s="22" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="D35" s="23" t="inlineStr">
-        <is>
-          <t>Explorateur : déplier le disque HERVE EDU (F:).</t>
-        </is>
-      </c>
-      <c r="E35" s="23" t="inlineStr">
-        <is>
-          <t>Les dossiers FOUND.000 à FOUND.004 n'apparaissent plus.</t>
-        </is>
-      </c>
-      <c r="F35" s="24" t="inlineStr">
+    <row r="40" ht="38.25" customHeight="1">
+      <c r="A40" s="18" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="19" t="inlineStr">
+        <is>
+          <t>E. SYNC</t>
+        </is>
+      </c>
+      <c r="C40" s="18" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="D40" s="19" t="inlineStr">
+        <is>
+          <t>SYNC : tous les rushes Panasonic sans LTC et tous les sons (tests compris), méthode Automatique.</t>
+        </is>
+      </c>
+      <c r="E40" s="19" t="inlineStr">
+        <is>
+          <t>Bon son pour chaque plan ; remarque « timecode sans rapport avec le son : son retrouvé par la forme d'onde » ; les sons de test restent non utilisés (mode AUDIO).</t>
+        </is>
+      </c>
+      <c r="F40" s="20" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="G35" s="24" t="inlineStr"/>
-      <c r="H35" s="25" t="n"/>
-      <c r="I35" s="26" t="inlineStr"/>
-      <c r="J35" s="27" t="inlineStr">
+      <c r="G40" s="20" t="n"/>
+      <c r="H40" s="21" t="n"/>
+      <c r="I40" s="22" t="n"/>
+      <c r="J40" s="23" t="inlineStr">
         <is>
           <t>Nouveau test (correctifs du 24/10).</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="22" t="n">
-        <v>32</v>
-      </c>
-      <c r="B36" s="23" t="inlineStr">
+    <row r="41" ht="38.25" customHeight="1">
+      <c r="A41" s="18" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="19" t="inlineStr">
+        <is>
+          <t>E. SYNC</t>
+        </is>
+      </c>
+      <c r="C41" s="18" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="D41" s="19" t="inlineStr">
+        <is>
+          <t>SYNC : créer les fichiers synchronisés (option « une piste mono par canal » cochée par défaut), puis les ouvrir dans Premiere.</t>
+        </is>
+      </c>
+      <c r="E41" s="19" t="inlineStr">
+        <is>
+          <t>Image présente ; 6 pistes mono de l'enregistreur + pistes caméra ; son calé sur le clap.</t>
+        </is>
+      </c>
+      <c r="F41" s="20" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="G41" s="20" t="n"/>
+      <c r="H41" s="21" t="n"/>
+      <c r="I41" s="22" t="n"/>
+      <c r="J41" s="23" t="inlineStr">
+        <is>
+          <t>Nouveau test (correctifs du 24/10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="29" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="30" t="inlineStr">
         <is>
           <t>D. PLAYER</t>
         </is>
       </c>
-      <c r="C36" s="22" t="inlineStr">
+      <c r="C42" s="29" t="inlineStr">
         <is>
           <t>38</t>
         </is>
       </c>
-      <c r="D36" s="23" t="inlineStr">
-        <is>
-          <t>PLAYER en mode AUDIO : cliquer SOLO puis MUTE sur une piste.</t>
-        </is>
-      </c>
-      <c r="E36" s="23" t="inlineStr">
-        <is>
-          <t>SOLO en orange, MUTE en rouge quand ils sont actifs.</t>
-        </is>
-      </c>
-      <c r="F36" s="24" t="inlineStr">
+      <c r="D42" s="30" t="inlineStr">
+        <is>
+          <t>PLAYER : sur une piste, cliquer S puis M (mode AUDIO et pistes d'une vidéo en mode VIDEO).</t>
+        </is>
+      </c>
+      <c r="E42" s="30" t="inlineStr">
+        <is>
+          <t>S orange, M rouge. Piste en S et en M : coupée. Bouton S présent sur chaque piste des vidéos.</t>
+        </is>
+      </c>
+      <c r="F42" s="31" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="G36" s="24" t="inlineStr"/>
-      <c r="H36" s="25" t="n"/>
-      <c r="I36" s="26" t="inlineStr"/>
-      <c r="J36" s="27" t="inlineStr">
-        <is>
-          <t>Nouveau test (correctifs du 24/10).</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="22" t="n">
-        <v>33</v>
-      </c>
-      <c r="B37" s="23" t="inlineStr">
+      <c r="G42" s="31" t="inlineStr"/>
+      <c r="H42" s="32" t="n"/>
+      <c r="I42" s="33" t="inlineStr"/>
+      <c r="J42" s="34" t="inlineStr">
+        <is>
+          <t>Nouveau test (correctifs du 26/10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="29" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" s="30" t="inlineStr">
         <is>
           <t>A. Installation et menus</t>
         </is>
       </c>
-      <c r="C37" s="22" t="inlineStr">
+      <c r="C43" s="29" t="inlineStr">
         <is>
           <t>38</t>
         </is>
       </c>
-      <c r="D37" s="23" t="inlineStr">
-        <is>
-          <t>Ouvrir un projet et regarder la barre du haut.</t>
-        </is>
-      </c>
-      <c r="E37" s="23" t="inlineStr">
-        <is>
-          <t>Nom du projet au centre de la fenêtre.</t>
-        </is>
-      </c>
-      <c r="F37" s="24" t="inlineStr">
+      <c r="D43" s="30" t="inlineStr">
+        <is>
+          <t>Lancer VERIFLOW pour la première fois après installation, puis le réduire en fenêtre, le fermer et le rouvrir.</t>
+        </is>
+      </c>
+      <c r="E43" s="30" t="inlineStr">
+        <is>
+          <t>Premier lancement : fenêtre agrandie à l'écran. Ensuite, VERIFLOW se rouvre comme tu l'as laissé (fenêtre ou agrandi).</t>
+        </is>
+      </c>
+      <c r="F43" s="31" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="G37" s="24" t="inlineStr"/>
-      <c r="H37" s="25" t="n"/>
-      <c r="I37" s="26" t="inlineStr"/>
-      <c r="J37" s="27" t="inlineStr">
-        <is>
-          <t>Nouveau test (correctifs du 24/10).</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="22" t="n">
-        <v>34</v>
-      </c>
-      <c r="B38" s="23" t="inlineStr">
-        <is>
-          <t>C. MEDIA et second écran</t>
-        </is>
-      </c>
-      <c r="C38" s="22" t="inlineStr">
-        <is>
-          <t>38</t>
-        </is>
-      </c>
-      <c r="D38" s="23" t="inlineStr">
-        <is>
-          <t>MEDIA : modifier un champ, puis Entrée (clavier principal), puis un autre avec Entrée du pavé numérique. Regarder la barre Enregistrer et la colonne TC en mode AUDIO.</t>
-        </is>
-      </c>
-      <c r="E38" s="23" t="inlineStr">
-        <is>
-          <t>Enregistré à chaque Entrée ; barre Enregistrer sur toute la largeur, séparée des champs ; TC affiché pour les WAV.</t>
-        </is>
-      </c>
-      <c r="F38" s="24" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G38" s="24" t="inlineStr"/>
-      <c r="H38" s="25" t="n"/>
-      <c r="I38" s="26" t="inlineStr"/>
-      <c r="J38" s="27" t="inlineStr">
-        <is>
-          <t>Nouveau test (correctifs du 24/10).</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="22" t="n">
-        <v>35</v>
-      </c>
-      <c r="B39" s="23" t="inlineStr">
-        <is>
-          <t>E. SYNC</t>
-        </is>
-      </c>
-      <c r="C39" s="22" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="D39" s="23" t="inlineStr">
-        <is>
-          <t>SYNC : un rush vidéo avec LTC sur une piste et son témoin sur l'autre, avec son WAV. Méthode Automatique, Analyser.</t>
-        </is>
-      </c>
-      <c r="E39" s="23" t="inlineStr">
-        <is>
-          <t>Colonne Méthode : LTC ; badge LTC à côté du timecode ; TC = celui du LTC (pas l'horloge de la Panasonic).</t>
-        </is>
-      </c>
-      <c r="F39" s="24" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G39" s="24" t="inlineStr"/>
-      <c r="H39" s="25" t="n"/>
-      <c r="I39" s="26" t="inlineStr"/>
-      <c r="J39" s="27" t="inlineStr">
-        <is>
-          <t>Nouveau test (correctifs du 24/10).</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="22" t="n">
-        <v>36</v>
-      </c>
-      <c r="B40" s="23" t="inlineStr">
-        <is>
-          <t>E. SYNC</t>
-        </is>
-      </c>
-      <c r="C40" s="22" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="D40" s="23" t="inlineStr">
-        <is>
-          <t>SYNC : tous les rushes Panasonic sans LTC et tous les sons (tests compris), méthode Automatique.</t>
-        </is>
-      </c>
-      <c r="E40" s="23" t="inlineStr">
-        <is>
-          <t>Bon son pour chaque plan ; remarque « timecode sans rapport avec le son : son retrouvé par la forme d'onde » ; les sons de test restent non utilisés (mode AUDIO).</t>
-        </is>
-      </c>
-      <c r="F40" s="24" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G40" s="24" t="inlineStr"/>
-      <c r="H40" s="25" t="n"/>
-      <c r="I40" s="26" t="inlineStr"/>
-      <c r="J40" s="27" t="inlineStr">
-        <is>
-          <t>Nouveau test (correctifs du 24/10).</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="22" t="n">
-        <v>37</v>
-      </c>
-      <c r="B41" s="23" t="inlineStr">
-        <is>
-          <t>E. SYNC</t>
-        </is>
-      </c>
-      <c r="C41" s="22" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="D41" s="23" t="inlineStr">
-        <is>
-          <t>SYNC : créer les fichiers synchronisés (option « une piste mono par canal » cochée par défaut), puis les ouvrir dans Premiere.</t>
-        </is>
-      </c>
-      <c r="E41" s="23" t="inlineStr">
-        <is>
-          <t>Image présente ; 6 pistes mono de l'enregistreur + pistes caméra ; son calé sur le clap.</t>
-        </is>
-      </c>
-      <c r="F41" s="24" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="G41" s="24" t="inlineStr"/>
-      <c r="H41" s="25" t="n"/>
-      <c r="I41" s="26" t="inlineStr"/>
-      <c r="J41" s="27" t="inlineStr">
-        <is>
-          <t>Nouveau test (correctifs du 24/10).</t>
+      <c r="G43" s="31" t="inlineStr"/>
+      <c r="H43" s="32" t="n"/>
+      <c r="I43" s="33" t="inlineStr"/>
+      <c r="J43" s="34" t="inlineStr">
+        <is>
+          <t>Nouveau test (correctifs du 26/10).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J41"/>
-  <conditionalFormatting sqref="G5:G41">
+  <autoFilter ref="A4:J43">
+    <filterColumn colId="6" hiddenButton="0" showButton="1">
+      <filters blank="1">
+        <filter val="KO"/>
+        <filter val="Partiel"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <conditionalFormatting sqref="G5:G43">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="6">
       <formula>"OK"</formula>
     </cfRule>
@@ -2425,13 +2606,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="F5:F41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F5:F43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Oui,Non"</formula1>
     </dataValidation>
-    <dataValidation sqref="G5:G41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,KO,Partiel,Non testable"</formula1>
     </dataValidation>
-    <dataValidation sqref="H5:H41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date" operator="greaterThan">
+    <dataValidation sqref="H5:H43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date" operator="greaterThan">
       <formula1>DATE(2026,1,1)</formula1>
     </dataValidation>
   </dataValidations>
@@ -2447,836 +2628,836 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="4" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="7" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="16.5" customHeight="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Synthèse (calculée automatiquement depuis l'onglet Tests)</t>
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
-      <c r="A3" s="28" t="inlineStr">
+      <c r="A3" s="24" t="inlineStr">
         <is>
           <t>PR</t>
         </is>
       </c>
-      <c r="B3" s="28" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>Tests</t>
         </is>
       </c>
-      <c r="C3" s="28" t="inlineStr">
+      <c r="C3" s="24" t="inlineStr">
         <is>
           <t>Effectués</t>
         </is>
       </c>
-      <c r="D3" s="28" t="inlineStr">
+      <c r="D3" s="24" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="E3" s="28" t="inlineStr">
+      <c r="E3" s="24" t="inlineStr">
         <is>
           <t>KO</t>
         </is>
       </c>
-      <c r="F3" s="28" t="inlineStr">
+      <c r="F3" s="24" t="inlineStr">
         <is>
           <t>Partiel</t>
         </is>
       </c>
-      <c r="G3" s="28" t="inlineStr">
+      <c r="G3" s="24" t="inlineStr">
         <is>
           <t>Non testable</t>
         </is>
       </c>
-      <c r="H3" s="28" t="inlineStr">
+      <c r="H3" s="24" t="inlineStr">
         <is>
           <t>Statut</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="29" t="inlineStr">
+      <c r="A4" s="25" t="inlineStr">
         <is>
           <t>17</t>
         </is>
       </c>
-      <c r="B4" s="29">
-        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A4&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C4" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A4&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D4" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A4&amp;"*",Tests!$G$5:$G$41,"OK")</f>
-        <v/>
-      </c>
-      <c r="E4" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A4&amp;"*",Tests!$G$5:$G$41,"KO")</f>
-        <v/>
-      </c>
-      <c r="F4" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A4&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G4" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A4&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H4" s="29">
+      <c r="B4" s="25">
+        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A4&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C4" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A4&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D4" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A4&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <v/>
+      </c>
+      <c r="E4" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A4&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <v/>
+      </c>
+      <c r="F4" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A4&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G4" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A4&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H4" s="25">
         <f>IF(E4&gt;0,"À corriger",IF(D4+G4=B4,"Validée",IF(C4=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="29" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="B5" s="29">
-        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A5&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C5" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A5&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D5" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A5&amp;"*",Tests!$G$5:$G$41,"OK")</f>
-        <v/>
-      </c>
-      <c r="E5" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A5&amp;"*",Tests!$G$5:$G$41,"KO")</f>
-        <v/>
-      </c>
-      <c r="F5" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A5&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G5" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A5&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H5" s="29">
+      <c r="B5" s="25">
+        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A5&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C5" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A5&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D5" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A5&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <v/>
+      </c>
+      <c r="E5" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A5&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <v/>
+      </c>
+      <c r="F5" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A5&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G5" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A5&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H5" s="25">
         <f>IF(E5&gt;0,"À corriger",IF(D5+G5=B5,"Validée",IF(C5=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="29" t="inlineStr">
+      <c r="A6" s="25" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="B6" s="29">
-        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A6&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C6" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A6&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D6" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A6&amp;"*",Tests!$G$5:$G$41,"OK")</f>
-        <v/>
-      </c>
-      <c r="E6" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A6&amp;"*",Tests!$G$5:$G$41,"KO")</f>
-        <v/>
-      </c>
-      <c r="F6" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A6&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G6" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A6&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H6" s="29">
+      <c r="B6" s="25">
+        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A6&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C6" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A6&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D6" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A6&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <v/>
+      </c>
+      <c r="E6" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A6&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <v/>
+      </c>
+      <c r="F6" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A6&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G6" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A6&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H6" s="25">
         <f>IF(E6&gt;0,"À corriger",IF(D6+G6=B6,"Validée",IF(C6=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="29" t="inlineStr">
+      <c r="A7" s="25" t="inlineStr">
         <is>
           <t>23</t>
         </is>
       </c>
-      <c r="B7" s="29">
-        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A7&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C7" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A7&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D7" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A7&amp;"*",Tests!$G$5:$G$41,"OK")</f>
-        <v/>
-      </c>
-      <c r="E7" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A7&amp;"*",Tests!$G$5:$G$41,"KO")</f>
-        <v/>
-      </c>
-      <c r="F7" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A7&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G7" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A7&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H7" s="29">
+      <c r="B7" s="25">
+        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A7&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C7" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A7&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D7" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A7&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <v/>
+      </c>
+      <c r="E7" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A7&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <v/>
+      </c>
+      <c r="F7" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A7&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G7" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A7&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H7" s="25">
         <f>IF(E7&gt;0,"À corriger",IF(D7+G7=B7,"Validée",IF(C7=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="29" t="inlineStr">
+      <c r="A8" s="25" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="B8" s="29">
-        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A8&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C8" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A8&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D8" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A8&amp;"*",Tests!$G$5:$G$41,"OK")</f>
-        <v/>
-      </c>
-      <c r="E8" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A8&amp;"*",Tests!$G$5:$G$41,"KO")</f>
-        <v/>
-      </c>
-      <c r="F8" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A8&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G8" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A8&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H8" s="29">
+      <c r="B8" s="25">
+        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A8&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C8" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A8&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D8" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A8&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <v/>
+      </c>
+      <c r="E8" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A8&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <v/>
+      </c>
+      <c r="F8" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A8&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G8" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A8&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H8" s="25">
         <f>IF(E8&gt;0,"À corriger",IF(D8+G8=B8,"Validée",IF(C8=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="29" t="inlineStr">
+      <c r="A9" s="25" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="B9" s="29">
-        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A9&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C9" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A9&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D9" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A9&amp;"*",Tests!$G$5:$G$41,"OK")</f>
-        <v/>
-      </c>
-      <c r="E9" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A9&amp;"*",Tests!$G$5:$G$41,"KO")</f>
-        <v/>
-      </c>
-      <c r="F9" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A9&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G9" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A9&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H9" s="29">
+      <c r="B9" s="25">
+        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A9&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C9" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A9&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D9" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A9&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <v/>
+      </c>
+      <c r="E9" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A9&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <v/>
+      </c>
+      <c r="F9" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A9&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G9" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A9&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H9" s="25">
         <f>IF(E9&gt;0,"À corriger",IF(D9+G9=B9,"Validée",IF(C9=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="29" t="inlineStr">
+      <c r="A10" s="25" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="B10" s="29">
-        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A10&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C10" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A10&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D10" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A10&amp;"*",Tests!$G$5:$G$41,"OK")</f>
-        <v/>
-      </c>
-      <c r="E10" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A10&amp;"*",Tests!$G$5:$G$41,"KO")</f>
-        <v/>
-      </c>
-      <c r="F10" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A10&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G10" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A10&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H10" s="29">
+      <c r="B10" s="25">
+        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A10&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C10" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A10&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D10" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A10&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <v/>
+      </c>
+      <c r="E10" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A10&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <v/>
+      </c>
+      <c r="F10" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A10&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G10" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A10&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H10" s="25">
         <f>IF(E10&gt;0,"À corriger",IF(D10+G10=B10,"Validée",IF(C10=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="29" t="inlineStr">
+      <c r="A11" s="25" t="inlineStr">
         <is>
           <t>27</t>
         </is>
       </c>
-      <c r="B11" s="29">
-        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A11&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C11" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A11&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D11" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A11&amp;"*",Tests!$G$5:$G$41,"OK")</f>
-        <v/>
-      </c>
-      <c r="E11" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A11&amp;"*",Tests!$G$5:$G$41,"KO")</f>
-        <v/>
-      </c>
-      <c r="F11" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A11&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G11" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A11&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H11" s="29">
+      <c r="B11" s="25">
+        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A11&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C11" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A11&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D11" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A11&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <v/>
+      </c>
+      <c r="E11" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A11&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <v/>
+      </c>
+      <c r="F11" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A11&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G11" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A11&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H11" s="25">
         <f>IF(E11&gt;0,"À corriger",IF(D11+G11=B11,"Validée",IF(C11=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="29" t="inlineStr">
+      <c r="A12" s="25" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="B12" s="29">
-        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A12&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C12" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A12&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D12" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A12&amp;"*",Tests!$G$5:$G$41,"OK")</f>
-        <v/>
-      </c>
-      <c r="E12" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A12&amp;"*",Tests!$G$5:$G$41,"KO")</f>
-        <v/>
-      </c>
-      <c r="F12" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A12&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G12" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A12&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H12" s="29">
+      <c r="B12" s="25">
+        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A12&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C12" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A12&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D12" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A12&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <v/>
+      </c>
+      <c r="E12" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A12&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <v/>
+      </c>
+      <c r="F12" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A12&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G12" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A12&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H12" s="25">
         <f>IF(E12&gt;0,"À corriger",IF(D12+G12=B12,"Validée",IF(C12=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="29" t="inlineStr">
+      <c r="A13" s="25" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="B13" s="29">
-        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A13&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C13" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A13&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D13" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A13&amp;"*",Tests!$G$5:$G$41,"OK")</f>
-        <v/>
-      </c>
-      <c r="E13" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A13&amp;"*",Tests!$G$5:$G$41,"KO")</f>
-        <v/>
-      </c>
-      <c r="F13" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A13&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G13" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A13&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H13" s="29">
+      <c r="B13" s="25">
+        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A13&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C13" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A13&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D13" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A13&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <v/>
+      </c>
+      <c r="E13" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A13&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <v/>
+      </c>
+      <c r="F13" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A13&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G13" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A13&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H13" s="25">
         <f>IF(E13&gt;0,"À corriger",IF(D13+G13=B13,"Validée",IF(C13=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="29" t="inlineStr">
+      <c r="A14" s="25" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="B14" s="29">
-        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A14&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C14" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A14&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D14" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A14&amp;"*",Tests!$G$5:$G$41,"OK")</f>
-        <v/>
-      </c>
-      <c r="E14" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A14&amp;"*",Tests!$G$5:$G$41,"KO")</f>
-        <v/>
-      </c>
-      <c r="F14" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A14&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G14" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A14&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H14" s="29">
+      <c r="B14" s="25">
+        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A14&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C14" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A14&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D14" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A14&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <v/>
+      </c>
+      <c r="E14" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A14&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <v/>
+      </c>
+      <c r="F14" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A14&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G14" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A14&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H14" s="25">
         <f>IF(E14&gt;0,"À corriger",IF(D14+G14=B14,"Validée",IF(C14=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="29" t="inlineStr">
+      <c r="A15" s="25" t="inlineStr">
         <is>
           <t>31</t>
         </is>
       </c>
-      <c r="B15" s="29">
-        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A15&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C15" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A15&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D15" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A15&amp;"*",Tests!$G$5:$G$41,"OK")</f>
-        <v/>
-      </c>
-      <c r="E15" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A15&amp;"*",Tests!$G$5:$G$41,"KO")</f>
-        <v/>
-      </c>
-      <c r="F15" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A15&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G15" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A15&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H15" s="29">
+      <c r="B15" s="25">
+        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A15&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C15" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A15&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D15" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A15&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <v/>
+      </c>
+      <c r="E15" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A15&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <v/>
+      </c>
+      <c r="F15" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A15&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G15" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A15&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H15" s="25">
         <f>IF(E15&gt;0,"À corriger",IF(D15+G15=B15,"Validée",IF(C15=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="29" t="inlineStr">
+      <c r="A16" s="25" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="B16" s="29">
-        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A16&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C16" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A16&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D16" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A16&amp;"*",Tests!$G$5:$G$41,"OK")</f>
-        <v/>
-      </c>
-      <c r="E16" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A16&amp;"*",Tests!$G$5:$G$41,"KO")</f>
-        <v/>
-      </c>
-      <c r="F16" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A16&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G16" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A16&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H16" s="29">
+      <c r="B16" s="25">
+        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A16&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C16" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A16&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D16" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A16&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <v/>
+      </c>
+      <c r="E16" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A16&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <v/>
+      </c>
+      <c r="F16" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A16&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G16" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A16&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H16" s="25">
         <f>IF(E16&gt;0,"À corriger",IF(D16+G16=B16,"Validée",IF(C16=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="29" t="inlineStr">
+      <c r="A17" s="25" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="B17" s="29">
-        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A17&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C17" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A17&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D17" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A17&amp;"*",Tests!$G$5:$G$41,"OK")</f>
-        <v/>
-      </c>
-      <c r="E17" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A17&amp;"*",Tests!$G$5:$G$41,"KO")</f>
-        <v/>
-      </c>
-      <c r="F17" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A17&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G17" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A17&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H17" s="29">
+      <c r="B17" s="25">
+        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A17&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C17" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A17&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D17" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A17&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <v/>
+      </c>
+      <c r="E17" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A17&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <v/>
+      </c>
+      <c r="F17" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A17&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G17" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A17&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H17" s="25">
         <f>IF(E17&gt;0,"À corriger",IF(D17+G17=B17,"Validée",IF(C17=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="29" t="inlineStr">
+      <c r="A18" s="25" t="inlineStr">
         <is>
           <t>34</t>
         </is>
       </c>
-      <c r="B18" s="29">
-        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A18&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C18" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A18&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D18" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A18&amp;"*",Tests!$G$5:$G$41,"OK")</f>
-        <v/>
-      </c>
-      <c r="E18" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A18&amp;"*",Tests!$G$5:$G$41,"KO")</f>
-        <v/>
-      </c>
-      <c r="F18" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A18&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G18" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A18&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H18" s="29">
+      <c r="B18" s="25">
+        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A18&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C18" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A18&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D18" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A18&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <v/>
+      </c>
+      <c r="E18" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A18&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <v/>
+      </c>
+      <c r="F18" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A18&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G18" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A18&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H18" s="25">
         <f>IF(E18&gt;0,"À corriger",IF(D18+G18=B18,"Validée",IF(C18=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="29" t="inlineStr">
+      <c r="A19" s="25" t="inlineStr">
         <is>
           <t>35</t>
         </is>
       </c>
-      <c r="B19" s="29">
-        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A19&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C19" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A19&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D19" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A19&amp;"*",Tests!$G$5:$G$41,"OK")</f>
-        <v/>
-      </c>
-      <c r="E19" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A19&amp;"*",Tests!$G$5:$G$41,"KO")</f>
-        <v/>
-      </c>
-      <c r="F19" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A19&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G19" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A19&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H19" s="29">
+      <c r="B19" s="25">
+        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A19&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C19" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A19&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D19" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A19&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <v/>
+      </c>
+      <c r="E19" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A19&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <v/>
+      </c>
+      <c r="F19" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A19&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G19" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A19&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H19" s="25">
         <f>IF(E19&gt;0,"À corriger",IF(D19+G19=B19,"Validée",IF(C19=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="29" t="inlineStr">
+      <c r="A20" s="25" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B20" s="29">
-        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A20&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C20" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A20&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D20" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A20&amp;"*",Tests!$G$5:$G$41,"OK")</f>
-        <v/>
-      </c>
-      <c r="E20" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A20&amp;"*",Tests!$G$5:$G$41,"KO")</f>
-        <v/>
-      </c>
-      <c r="F20" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A20&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G20" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A20&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H20" s="29">
+      <c r="B20" s="25">
+        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A20&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C20" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A20&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D20" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A20&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <v/>
+      </c>
+      <c r="E20" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A20&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <v/>
+      </c>
+      <c r="F20" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A20&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G20" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A20&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H20" s="25">
         <f>IF(E20&gt;0,"À corriger",IF(D20+G20=B20,"Validée",IF(C20=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="29" t="inlineStr">
+      <c r="A21" s="25" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="B21" s="29">
-        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A21&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C21" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A21&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D21" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A21&amp;"*",Tests!$G$5:$G$41,"OK")</f>
-        <v/>
-      </c>
-      <c r="E21" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A21&amp;"*",Tests!$G$5:$G$41,"KO")</f>
-        <v/>
-      </c>
-      <c r="F21" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A21&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G21" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A21&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H21" s="29">
+      <c r="B21" s="25">
+        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A21&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C21" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A21&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D21" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A21&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <v/>
+      </c>
+      <c r="E21" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A21&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <v/>
+      </c>
+      <c r="F21" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A21&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G21" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A21&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H21" s="25">
         <f>IF(E21&gt;0,"À corriger",IF(D21+G21=B21,"Validée",IF(C21=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="29" t="inlineStr">
+      <c r="A22" s="25" t="inlineStr">
         <is>
           <t>38</t>
         </is>
       </c>
-      <c r="B22" s="29">
-        <f>COUNTIF(Tests!$C$5:$C$41,"*"&amp;A22&amp;"*")</f>
-        <v/>
-      </c>
-      <c r="C22" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A22&amp;"*",Tests!$F$5:$F$41,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D22" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A22&amp;"*",Tests!$G$5:$G$41,"OK")</f>
-        <v/>
-      </c>
-      <c r="E22" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A22&amp;"*",Tests!$G$5:$G$41,"KO")</f>
-        <v/>
-      </c>
-      <c r="F22" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A22&amp;"*",Tests!$G$5:$G$41,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G22" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,"*"&amp;A22&amp;"*",Tests!$G$5:$G$41,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H22" s="29">
+      <c r="B22" s="25">
+        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A22&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="C22" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A22&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D22" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A22&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <v/>
+      </c>
+      <c r="E22" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A22&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <v/>
+      </c>
+      <c r="F22" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A22&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G22" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A22&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H22" s="25">
         <f>IF(E22&gt;0,"À corriger",IF(D22+G22=B22,"Validée",IF(C22=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="29" t="inlineStr">
+      <c r="A23" s="25" t="inlineStr">
         <is>
           <t>5 (en attente)</t>
         </is>
       </c>
-      <c r="B23" s="29">
-        <f>COUNTIF(Tests!$C$5:$C$41,A23)</f>
-        <v/>
-      </c>
-      <c r="C23" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,A23,Tests!$F$5:$F$41,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D23" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,A23,Tests!$G$5:$G$41,"OK")</f>
-        <v/>
-      </c>
-      <c r="E23" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,A23,Tests!$G$5:$G$41,"KO")</f>
-        <v/>
-      </c>
-      <c r="F23" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,A23,Tests!$G$5:$G$41,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G23" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,A23,Tests!$G$5:$G$41,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H23" s="29">
+      <c r="B23" s="25">
+        <f>COUNTIF(Tests!$C$5:$C$43,A23)</f>
+        <v/>
+      </c>
+      <c r="C23" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,A23,Tests!$F$5:$F$43,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D23" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,A23,Tests!$G$5:$G$43,"OK")</f>
+        <v/>
+      </c>
+      <c r="E23" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,A23,Tests!$G$5:$G$43,"KO")</f>
+        <v/>
+      </c>
+      <c r="F23" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,A23,Tests!$G$5:$G$43,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G23" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,A23,Tests!$G$5:$G$43,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H23" s="25">
         <f>IF(E23&gt;0,"À corriger",IF(D23+G23=B23,"Validée",IF(C23=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="29" t="inlineStr">
+      <c r="A24" s="25" t="inlineStr">
         <is>
           <t>SYNC</t>
         </is>
       </c>
-      <c r="B24" s="29">
-        <f>COUNTIF(Tests!$C$5:$C$41,A24)</f>
-        <v/>
-      </c>
-      <c r="C24" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,A24,Tests!$F$5:$F$41,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D24" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,A24,Tests!$G$5:$G$41,"OK")</f>
-        <v/>
-      </c>
-      <c r="E24" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,A24,Tests!$G$5:$G$41,"KO")</f>
-        <v/>
-      </c>
-      <c r="F24" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,A24,Tests!$G$5:$G$41,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G24" s="29">
-        <f>COUNTIFS(Tests!$C$5:$C$41,A24,Tests!$G$5:$G$41,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H24" s="29">
+      <c r="B24" s="25">
+        <f>COUNTIF(Tests!$C$5:$C$43,A24)</f>
+        <v/>
+      </c>
+      <c r="C24" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,A24,Tests!$F$5:$F$43,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D24" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,A24,Tests!$G$5:$G$43,"OK")</f>
+        <v/>
+      </c>
+      <c r="E24" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,A24,Tests!$G$5:$G$43,"KO")</f>
+        <v/>
+      </c>
+      <c r="F24" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,A24,Tests!$G$5:$G$43,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G24" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$43,A24,Tests!$G$5:$G$43,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H24" s="25">
         <f>IF(E24&gt;0,"À corriger",IF(D24+G24=B24,"Validée",IF(C24=0,"À tester","En cours")))</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="30" t="inlineStr">
+      <c r="A25" s="26" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B25" s="30">
-        <f>COUNTA(Tests!$A$5:$A$41)</f>
-        <v/>
-      </c>
-      <c r="C25" s="30">
-        <f>COUNTIF(Tests!$F$5:$F$41,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D25" s="30">
-        <f>COUNTIF(Tests!$G$5:$G$41,"OK")</f>
-        <v/>
-      </c>
-      <c r="E25" s="30">
-        <f>COUNTIF(Tests!$G$5:$G$41,"KO")</f>
-        <v/>
-      </c>
-      <c r="F25" s="30">
-        <f>COUNTIF(Tests!$G$5:$G$41,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G25" s="30">
-        <f>COUNTIF(Tests!$G$5:$G$41,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H25" s="30" t="n"/>
-    </row>
+      <c r="B25" s="26">
+        <f>COUNTA(Tests!$A$5:$A$43)</f>
+        <v/>
+      </c>
+      <c r="C25" s="26">
+        <f>COUNTIF(Tests!$F$5:$F$43,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D25" s="26">
+        <f>COUNTIF(Tests!$G$5:$G$43,"OK")</f>
+        <v/>
+      </c>
+      <c r="E25" s="26">
+        <f>COUNTIF(Tests!$G$5:$G$43,"KO")</f>
+        <v/>
+      </c>
+      <c r="F25" s="26">
+        <f>COUNTIF(Tests!$G$5:$G$43,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G25" s="26">
+        <f>COUNTIF(Tests!$G$5:$G$43,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H25" s="26" t="n"/>
+    </row>
+    <row r="26"/>
     <row r="27">
-      <c r="A27" s="31" t="inlineStr">
+      <c r="A27" s="27" t="inlineStr">
         <is>
           <t>Un test peut couvrir plusieurs PR : il compte pour chacune. « Validée » = tous les tests de la PR en OK ou Non testable. Un test « Partiel » corrigé depuis reste « En cours » jusqu'à ce que tu le refasses.</t>
         </is>
@@ -3284,10 +3465,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="H4:H24">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="6">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="1">
       <formula>"Validée"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="7">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="0">
       <formula>"À corriger"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3318,96 +3499,96 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="14" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>Cellules à remplir</t>
         </is>
       </c>
-      <c r="B2" s="15" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>Colonnes jaunes de l'onglet Tests : Effectué, Résultat, Date, Commentaires. Le reste est fixe.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Effectué</t>
         </is>
       </c>
-      <c r="B3" s="15" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Oui ou Non (liste déroulante).</t>
         </is>
       </c>
     </row>
     <row r="4" ht="25.5" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Résultat</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>OK : conforme au résultat attendu. KO : non conforme. Partiel : en partie conforme (préciser). Non testable : matériel ou fichier absent.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>Date du test, format JJ/MM/AAAA.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="25.5" customHeight="1">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Commentaires</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Pour un KO ou un Partiel : ce qui s'est passé, le message affiché, le fichier utilisé (format, caméra, codec).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Ordre</t>
         </is>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Suivre l'ordre des numéros. La section G (désinstallation) efface les réglages : la faire en dernier.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="14" t="inlineStr">
+    <row r="8" ht="25.5" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Build</t>
         </is>
       </c>
-      <c r="B8" s="15" t="inlineStr">
-        <is>
-          <t>https://github.com/Herve-obe/VERIFLOW-v4/actions/runs/40104706786 (artefact veriflow-windows-latest, build du 24/10).</t>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>https://github.com/Herve-obe/VERIFLOW-v4/actions/runs/40517638115 (artefact veriflow-windows-latest, build du 27/10).</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Retour</t>
         </is>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Déposer le fichier rempli dans la conversation, ou le pousser dans docs/recette/ du dépôt.</t>
         </is>
@@ -3422,62 +3603,62 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>N°</t>
         </is>
       </c>
-      <c r="B12" s="16" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>PR</t>
         </is>
       </c>
-      <c r="C12" s="16" t="inlineStr">
+      <c r="C12" s="12" t="inlineStr">
         <is>
           <t>Effectué</t>
         </is>
       </c>
-      <c r="D12" s="16" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>Résultat</t>
         </is>
       </c>
-      <c r="E12" s="16" t="inlineStr">
+      <c r="E12" s="12" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="F12" s="16" t="inlineStr">
+      <c r="F12" s="12" t="inlineStr">
         <is>
           <t>Commentaires</t>
         </is>
       </c>
     </row>
     <row r="13" ht="25.5" customHeight="1">
-      <c r="A13" s="17" t="n">
+      <c r="A13" s="13" t="n">
         <v>13</v>
       </c>
-      <c r="B13" s="17" t="inlineStr">
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="C13" s="17" t="inlineStr">
+      <c r="C13" s="13" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="D13" s="17" t="inlineStr">
+      <c r="D13" s="13" t="inlineStr">
         <is>
           <t>KO</t>
         </is>
       </c>
-      <c r="E13" s="17" t="inlineStr">
+      <c r="E13" s="13" t="inlineStr">
         <is>
           <t>21/10/2026</t>
         </is>
       </c>
-      <c r="F13" s="17" t="inlineStr">
+      <c r="F13" s="13" t="inlineStr">
         <is>
           <t>Fichier ouvert dans Reaper : message affiché, mais le disque a disparu de l'explorateur.</t>
         </is>

</xml_diff>

<commit_message>
Recette : tests 40 à 42 (PR 39, carte réutilisée, veille, débit)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MoqekrFvgrWkuAe5NHnE5A
</commit_message>
<xml_diff>
--- a/docs/recette/RECETTE_PR_17-37.xlsx
+++ b/docs/recette/RECETTE_PR_17-37.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Légende" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tests'!$A$4:$J$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tests'!$A$4:$J$46</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Tests'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -749,7 +749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -766,7 +766,7 @@
     <row r="1" ht="18" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Recette VERIFLOW : PR 17 à 38 (build de la branche claude/recette, Windows 11)</t>
+          <t>Recette VERIFLOW : PR 17 à 39 (build de la branche claude/recette, Windows 11)</t>
         </is>
       </c>
     </row>
@@ -2582,8 +2582,122 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" s="29" t="n">
+        <v>40</v>
+      </c>
+      <c r="B44" s="30" t="inlineStr">
+        <is>
+          <t>C. OFFLOAD</t>
+        </is>
+      </c>
+      <c r="C44" s="29" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="D44" s="30" t="inlineStr">
+        <is>
+          <t>OFFLOAD dans un projet, modèle « {jour}/{carte} », jour J01 : copier une carte SD. Tourner quelques plans de plus sur la même carte sans la formater, puis relancer l'offload avec le jour J02.</t>
+        </is>
+      </c>
+      <c r="E44" s="30" t="inlineStr">
+        <is>
+          <t>Avant copie : message indiquant que des rushes de cette carte sont déjà copiés dans J01, avec « Reprendre dans ce dossier ». En le choisissant puis « Compléter la copie » : seuls les nouveaux plans sont copiés, les autres revérifiés. « Effacer et tout recopier » recopie toute la carte.</t>
+        </is>
+      </c>
+      <c r="F44" s="31" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="G44" s="31" t="n"/>
+      <c r="H44" s="32" t="n"/>
+      <c r="I44" s="33" t="n"/>
+      <c r="J44" s="34" t="inlineStr">
+        <is>
+          <t>Nouveau test (PR 39, 31/10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="29" t="n">
+        <v>41</v>
+      </c>
+      <c r="B45" s="30" t="inlineStr">
+        <is>
+          <t>C. OFFLOAD</t>
+        </is>
+      </c>
+      <c r="C45" s="29" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="D45" s="30" t="inlineStr">
+        <is>
+          <t>PC portable sur batterie, mise en veille réglée à 1 ou 2 minutes : lancer un offload qui dure plus longtemps, sans toucher au PC.</t>
+        </is>
+      </c>
+      <c r="E45" s="30" t="inlineStr">
+        <is>
+          <t>Le PC ne se met pas en veille pendant la copie (l'écran peut s'éteindre). Une fois la copie finie, la mise en veille revient normalement.</t>
+        </is>
+      </c>
+      <c r="F45" s="31" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="G45" s="31" t="n"/>
+      <c r="H45" s="32" t="n"/>
+      <c r="I45" s="33" t="n"/>
+      <c r="J45" s="34" t="inlineStr">
+        <is>
+          <t>Nouveau test (PR 39, 31/10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="29" t="n">
+        <v>42</v>
+      </c>
+      <c r="B46" s="30" t="inlineStr">
+        <is>
+          <t>C. OFFLOAD</t>
+        </is>
+      </c>
+      <c r="C46" s="29" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="D46" s="30" t="inlineStr">
+        <is>
+          <t>OFFLOAD d'une carte d'au moins 20 Go avec XXH128 seul, puis la même carte avec XXH128 + SHA-256. Noter le débit affiché et la durée totale.</t>
+        </is>
+      </c>
+      <c r="E46" s="30" t="inlineStr">
+        <is>
+          <t>Écart de durée faible entre les deux (la SHA-256 se calcule en parallèle de la lecture). Noter les deux durées dans Commentaires.</t>
+        </is>
+      </c>
+      <c r="F46" s="31" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="G46" s="31" t="n"/>
+      <c r="H46" s="32" t="n"/>
+      <c r="I46" s="33" t="n"/>
+      <c r="J46" s="34" t="inlineStr">
+        <is>
+          <t>Nouveau test (PR 39, 31/10).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:J43">
+  <autoFilter ref="A4:J46">
     <filterColumn colId="6" hiddenButton="0" showButton="1">
       <filters blank="1">
         <filter val="KO"/>
@@ -2591,7 +2705,7 @@
       </filters>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="G5:G43">
+  <conditionalFormatting sqref="G5:G46">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="6">
       <formula>"OK"</formula>
     </cfRule>
@@ -2606,13 +2720,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="F5:F43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F5:F46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Oui,Non"</formula1>
     </dataValidation>
-    <dataValidation sqref="G5:G43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,KO,Partiel,Non testable"</formula1>
     </dataValidation>
-    <dataValidation sqref="H5:H43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date" operator="greaterThan">
+    <dataValidation sqref="H5:H46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date" operator="greaterThan">
       <formula1>DATE(2026,1,1)</formula1>
     </dataValidation>
   </dataValidations>
@@ -2627,7 +2741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2645,7 +2759,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="24" t="inlineStr">
         <is>
@@ -2695,27 +2808,27 @@
         </is>
       </c>
       <c r="B4" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A4&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A4&amp;"*")</f>
         <v/>
       </c>
       <c r="C4" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A4&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A4&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
         <v/>
       </c>
       <c r="D4" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A4&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A4&amp;"*",Tests!$G$5:$G$46,"OK")</f>
         <v/>
       </c>
       <c r="E4" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A4&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A4&amp;"*",Tests!$G$5:$G$46,"KO")</f>
         <v/>
       </c>
       <c r="F4" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A4&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A4&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
         <v/>
       </c>
       <c r="G4" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A4&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A4&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
         <v/>
       </c>
       <c r="H4" s="25">
@@ -2730,27 +2843,27 @@
         </is>
       </c>
       <c r="B5" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A5&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A5&amp;"*")</f>
         <v/>
       </c>
       <c r="C5" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A5&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A5&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
         <v/>
       </c>
       <c r="D5" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A5&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A5&amp;"*",Tests!$G$5:$G$46,"OK")</f>
         <v/>
       </c>
       <c r="E5" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A5&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A5&amp;"*",Tests!$G$5:$G$46,"KO")</f>
         <v/>
       </c>
       <c r="F5" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A5&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A5&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
         <v/>
       </c>
       <c r="G5" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A5&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A5&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
         <v/>
       </c>
       <c r="H5" s="25">
@@ -2765,27 +2878,27 @@
         </is>
       </c>
       <c r="B6" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A6&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A6&amp;"*")</f>
         <v/>
       </c>
       <c r="C6" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A6&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A6&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
         <v/>
       </c>
       <c r="D6" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A6&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A6&amp;"*",Tests!$G$5:$G$46,"OK")</f>
         <v/>
       </c>
       <c r="E6" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A6&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A6&amp;"*",Tests!$G$5:$G$46,"KO")</f>
         <v/>
       </c>
       <c r="F6" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A6&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A6&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
         <v/>
       </c>
       <c r="G6" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A6&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A6&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
         <v/>
       </c>
       <c r="H6" s="25">
@@ -2800,27 +2913,27 @@
         </is>
       </c>
       <c r="B7" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A7&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A7&amp;"*")</f>
         <v/>
       </c>
       <c r="C7" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A7&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A7&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
         <v/>
       </c>
       <c r="D7" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A7&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A7&amp;"*",Tests!$G$5:$G$46,"OK")</f>
         <v/>
       </c>
       <c r="E7" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A7&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A7&amp;"*",Tests!$G$5:$G$46,"KO")</f>
         <v/>
       </c>
       <c r="F7" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A7&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A7&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
         <v/>
       </c>
       <c r="G7" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A7&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A7&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
         <v/>
       </c>
       <c r="H7" s="25">
@@ -2835,27 +2948,27 @@
         </is>
       </c>
       <c r="B8" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A8&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A8&amp;"*")</f>
         <v/>
       </c>
       <c r="C8" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A8&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A8&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
         <v/>
       </c>
       <c r="D8" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A8&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A8&amp;"*",Tests!$G$5:$G$46,"OK")</f>
         <v/>
       </c>
       <c r="E8" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A8&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A8&amp;"*",Tests!$G$5:$G$46,"KO")</f>
         <v/>
       </c>
       <c r="F8" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A8&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A8&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
         <v/>
       </c>
       <c r="G8" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A8&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A8&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
         <v/>
       </c>
       <c r="H8" s="25">
@@ -2870,27 +2983,27 @@
         </is>
       </c>
       <c r="B9" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A9&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A9&amp;"*")</f>
         <v/>
       </c>
       <c r="C9" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A9&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A9&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
         <v/>
       </c>
       <c r="D9" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A9&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A9&amp;"*",Tests!$G$5:$G$46,"OK")</f>
         <v/>
       </c>
       <c r="E9" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A9&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A9&amp;"*",Tests!$G$5:$G$46,"KO")</f>
         <v/>
       </c>
       <c r="F9" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A9&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A9&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
         <v/>
       </c>
       <c r="G9" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A9&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A9&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
         <v/>
       </c>
       <c r="H9" s="25">
@@ -2905,27 +3018,27 @@
         </is>
       </c>
       <c r="B10" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A10&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A10&amp;"*")</f>
         <v/>
       </c>
       <c r="C10" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A10&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A10&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
         <v/>
       </c>
       <c r="D10" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A10&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A10&amp;"*",Tests!$G$5:$G$46,"OK")</f>
         <v/>
       </c>
       <c r="E10" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A10&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A10&amp;"*",Tests!$G$5:$G$46,"KO")</f>
         <v/>
       </c>
       <c r="F10" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A10&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A10&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
         <v/>
       </c>
       <c r="G10" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A10&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A10&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
         <v/>
       </c>
       <c r="H10" s="25">
@@ -2940,27 +3053,27 @@
         </is>
       </c>
       <c r="B11" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A11&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A11&amp;"*")</f>
         <v/>
       </c>
       <c r="C11" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A11&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A11&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
         <v/>
       </c>
       <c r="D11" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A11&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A11&amp;"*",Tests!$G$5:$G$46,"OK")</f>
         <v/>
       </c>
       <c r="E11" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A11&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A11&amp;"*",Tests!$G$5:$G$46,"KO")</f>
         <v/>
       </c>
       <c r="F11" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A11&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A11&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
         <v/>
       </c>
       <c r="G11" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A11&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A11&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
         <v/>
       </c>
       <c r="H11" s="25">
@@ -2975,27 +3088,27 @@
         </is>
       </c>
       <c r="B12" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A12&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A12&amp;"*")</f>
         <v/>
       </c>
       <c r="C12" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A12&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A12&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
         <v/>
       </c>
       <c r="D12" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A12&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A12&amp;"*",Tests!$G$5:$G$46,"OK")</f>
         <v/>
       </c>
       <c r="E12" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A12&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A12&amp;"*",Tests!$G$5:$G$46,"KO")</f>
         <v/>
       </c>
       <c r="F12" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A12&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A12&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
         <v/>
       </c>
       <c r="G12" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A12&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A12&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
         <v/>
       </c>
       <c r="H12" s="25">
@@ -3010,27 +3123,27 @@
         </is>
       </c>
       <c r="B13" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A13&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A13&amp;"*")</f>
         <v/>
       </c>
       <c r="C13" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A13&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A13&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
         <v/>
       </c>
       <c r="D13" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A13&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A13&amp;"*",Tests!$G$5:$G$46,"OK")</f>
         <v/>
       </c>
       <c r="E13" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A13&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A13&amp;"*",Tests!$G$5:$G$46,"KO")</f>
         <v/>
       </c>
       <c r="F13" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A13&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A13&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
         <v/>
       </c>
       <c r="G13" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A13&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A13&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
         <v/>
       </c>
       <c r="H13" s="25">
@@ -3045,27 +3158,27 @@
         </is>
       </c>
       <c r="B14" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A14&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A14&amp;"*")</f>
         <v/>
       </c>
       <c r="C14" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A14&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A14&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
         <v/>
       </c>
       <c r="D14" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A14&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A14&amp;"*",Tests!$G$5:$G$46,"OK")</f>
         <v/>
       </c>
       <c r="E14" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A14&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A14&amp;"*",Tests!$G$5:$G$46,"KO")</f>
         <v/>
       </c>
       <c r="F14" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A14&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A14&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
         <v/>
       </c>
       <c r="G14" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A14&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A14&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
         <v/>
       </c>
       <c r="H14" s="25">
@@ -3080,27 +3193,27 @@
         </is>
       </c>
       <c r="B15" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A15&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A15&amp;"*")</f>
         <v/>
       </c>
       <c r="C15" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A15&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A15&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
         <v/>
       </c>
       <c r="D15" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A15&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A15&amp;"*",Tests!$G$5:$G$46,"OK")</f>
         <v/>
       </c>
       <c r="E15" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A15&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A15&amp;"*",Tests!$G$5:$G$46,"KO")</f>
         <v/>
       </c>
       <c r="F15" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A15&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A15&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
         <v/>
       </c>
       <c r="G15" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A15&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A15&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
         <v/>
       </c>
       <c r="H15" s="25">
@@ -3115,27 +3228,27 @@
         </is>
       </c>
       <c r="B16" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A16&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A16&amp;"*")</f>
         <v/>
       </c>
       <c r="C16" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A16&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A16&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
         <v/>
       </c>
       <c r="D16" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A16&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A16&amp;"*",Tests!$G$5:$G$46,"OK")</f>
         <v/>
       </c>
       <c r="E16" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A16&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A16&amp;"*",Tests!$G$5:$G$46,"KO")</f>
         <v/>
       </c>
       <c r="F16" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A16&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A16&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
         <v/>
       </c>
       <c r="G16" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A16&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A16&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
         <v/>
       </c>
       <c r="H16" s="25">
@@ -3150,27 +3263,27 @@
         </is>
       </c>
       <c r="B17" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A17&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A17&amp;"*")</f>
         <v/>
       </c>
       <c r="C17" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A17&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A17&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
         <v/>
       </c>
       <c r="D17" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A17&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A17&amp;"*",Tests!$G$5:$G$46,"OK")</f>
         <v/>
       </c>
       <c r="E17" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A17&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A17&amp;"*",Tests!$G$5:$G$46,"KO")</f>
         <v/>
       </c>
       <c r="F17" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A17&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A17&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
         <v/>
       </c>
       <c r="G17" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A17&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A17&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
         <v/>
       </c>
       <c r="H17" s="25">
@@ -3185,27 +3298,27 @@
         </is>
       </c>
       <c r="B18" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A18&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A18&amp;"*")</f>
         <v/>
       </c>
       <c r="C18" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A18&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A18&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
         <v/>
       </c>
       <c r="D18" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A18&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A18&amp;"*",Tests!$G$5:$G$46,"OK")</f>
         <v/>
       </c>
       <c r="E18" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A18&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A18&amp;"*",Tests!$G$5:$G$46,"KO")</f>
         <v/>
       </c>
       <c r="F18" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A18&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A18&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
         <v/>
       </c>
       <c r="G18" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A18&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A18&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
         <v/>
       </c>
       <c r="H18" s="25">
@@ -3220,27 +3333,27 @@
         </is>
       </c>
       <c r="B19" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A19&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A19&amp;"*")</f>
         <v/>
       </c>
       <c r="C19" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A19&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A19&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
         <v/>
       </c>
       <c r="D19" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A19&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A19&amp;"*",Tests!$G$5:$G$46,"OK")</f>
         <v/>
       </c>
       <c r="E19" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A19&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A19&amp;"*",Tests!$G$5:$G$46,"KO")</f>
         <v/>
       </c>
       <c r="F19" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A19&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A19&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
         <v/>
       </c>
       <c r="G19" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A19&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A19&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
         <v/>
       </c>
       <c r="H19" s="25">
@@ -3255,27 +3368,27 @@
         </is>
       </c>
       <c r="B20" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A20&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A20&amp;"*")</f>
         <v/>
       </c>
       <c r="C20" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A20&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A20&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
         <v/>
       </c>
       <c r="D20" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A20&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A20&amp;"*",Tests!$G$5:$G$46,"OK")</f>
         <v/>
       </c>
       <c r="E20" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A20&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A20&amp;"*",Tests!$G$5:$G$46,"KO")</f>
         <v/>
       </c>
       <c r="F20" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A20&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A20&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
         <v/>
       </c>
       <c r="G20" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A20&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A20&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
         <v/>
       </c>
       <c r="H20" s="25">
@@ -3290,27 +3403,27 @@
         </is>
       </c>
       <c r="B21" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A21&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A21&amp;"*")</f>
         <v/>
       </c>
       <c r="C21" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A21&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A21&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
         <v/>
       </c>
       <c r="D21" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A21&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A21&amp;"*",Tests!$G$5:$G$46,"OK")</f>
         <v/>
       </c>
       <c r="E21" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A21&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A21&amp;"*",Tests!$G$5:$G$46,"KO")</f>
         <v/>
       </c>
       <c r="F21" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A21&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A21&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
         <v/>
       </c>
       <c r="G21" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A21&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A21&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
         <v/>
       </c>
       <c r="H21" s="25">
@@ -3325,27 +3438,27 @@
         </is>
       </c>
       <c r="B22" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$43,"*"&amp;A22&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A22&amp;"*")</f>
         <v/>
       </c>
       <c r="C22" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A22&amp;"*",Tests!$F$5:$F$43,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A22&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
         <v/>
       </c>
       <c r="D22" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A22&amp;"*",Tests!$G$5:$G$43,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A22&amp;"*",Tests!$G$5:$G$46,"OK")</f>
         <v/>
       </c>
       <c r="E22" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A22&amp;"*",Tests!$G$5:$G$43,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A22&amp;"*",Tests!$G$5:$G$46,"KO")</f>
         <v/>
       </c>
       <c r="F22" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A22&amp;"*",Tests!$G$5:$G$43,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A22&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
         <v/>
       </c>
       <c r="G22" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,"*"&amp;A22&amp;"*",Tests!$G$5:$G$43,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A22&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
         <v/>
       </c>
       <c r="H22" s="25">
@@ -3356,31 +3469,31 @@
     <row r="23">
       <c r="A23" s="25" t="inlineStr">
         <is>
-          <t>5 (en attente)</t>
+          <t>39</t>
         </is>
       </c>
       <c r="B23" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$43,A23)</f>
+        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A23&amp;"*")</f>
         <v/>
       </c>
       <c r="C23" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,A23,Tests!$F$5:$F$43,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A23&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
         <v/>
       </c>
       <c r="D23" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,A23,Tests!$G$5:$G$43,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A23&amp;"*",Tests!$G$5:$G$46,"OK")</f>
         <v/>
       </c>
       <c r="E23" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,A23,Tests!$G$5:$G$43,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A23&amp;"*",Tests!$G$5:$G$46,"KO")</f>
         <v/>
       </c>
       <c r="F23" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,A23,Tests!$G$5:$G$43,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A23&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
         <v/>
       </c>
       <c r="G23" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,A23,Tests!$G$5:$G$43,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A23&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
         <v/>
       </c>
       <c r="H23" s="25">
@@ -3391,31 +3504,31 @@
     <row r="24">
       <c r="A24" s="25" t="inlineStr">
         <is>
-          <t>SYNC</t>
+          <t>5 (en attente)</t>
         </is>
       </c>
       <c r="B24" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$43,A24)</f>
+        <f>COUNTIF(Tests!$C$5:$C$46,A24)</f>
         <v/>
       </c>
       <c r="C24" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,A24,Tests!$F$5:$F$43,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,A24,Tests!$F$5:$F$46,"Oui")</f>
         <v/>
       </c>
       <c r="D24" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,A24,Tests!$G$5:$G$43,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,A24,Tests!$G$5:$G$46,"OK")</f>
         <v/>
       </c>
       <c r="E24" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,A24,Tests!$G$5:$G$43,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,A24,Tests!$G$5:$G$46,"KO")</f>
         <v/>
       </c>
       <c r="F24" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,A24,Tests!$G$5:$G$43,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,A24,Tests!$G$5:$G$46,"Partiel")</f>
         <v/>
       </c>
       <c r="G24" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$43,A24,Tests!$G$5:$G$43,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$46,A24,Tests!$G$5:$G$46,"Non testable")</f>
         <v/>
       </c>
       <c r="H24" s="25">
@@ -3424,47 +3537,82 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="26" t="inlineStr">
+      <c r="A25" s="25" t="inlineStr">
+        <is>
+          <t>SYNC</t>
+        </is>
+      </c>
+      <c r="B25" s="25">
+        <f>COUNTIF(Tests!$C$5:$C$46,A25)</f>
+        <v/>
+      </c>
+      <c r="C25" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$46,A25,Tests!$F$5:$F$46,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D25" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$46,A25,Tests!$G$5:$G$46,"OK")</f>
+        <v/>
+      </c>
+      <c r="E25" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$46,A25,Tests!$G$5:$G$46,"KO")</f>
+        <v/>
+      </c>
+      <c r="F25" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$46,A25,Tests!$G$5:$G$46,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G25" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$46,A25,Tests!$G$5:$G$46,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H25" s="25">
+        <f>IF(E25&gt;0,"À corriger",IF(D25+G25=B25,"Validée",IF(C25=0,"À tester","En cours")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="26" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B25" s="26">
-        <f>COUNTA(Tests!$A$5:$A$43)</f>
-        <v/>
-      </c>
-      <c r="C25" s="26">
-        <f>COUNTIF(Tests!$F$5:$F$43,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D25" s="26">
-        <f>COUNTIF(Tests!$G$5:$G$43,"OK")</f>
-        <v/>
-      </c>
-      <c r="E25" s="26">
-        <f>COUNTIF(Tests!$G$5:$G$43,"KO")</f>
-        <v/>
-      </c>
-      <c r="F25" s="26">
-        <f>COUNTIF(Tests!$G$5:$G$43,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G25" s="26">
-        <f>COUNTIF(Tests!$G$5:$G$43,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H25" s="26" t="n"/>
-    </row>
-    <row r="26"/>
-    <row r="27">
-      <c r="A27" s="27" t="inlineStr">
+      <c r="B26" s="26">
+        <f>COUNTA(Tests!$A$5:$A$46)</f>
+        <v/>
+      </c>
+      <c r="C26" s="26">
+        <f>COUNTIF(Tests!$F$5:$F$46,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D26" s="26">
+        <f>COUNTIF(Tests!$G$5:$G$46,"OK")</f>
+        <v/>
+      </c>
+      <c r="E26" s="26">
+        <f>COUNTIF(Tests!$G$5:$G$46,"KO")</f>
+        <v/>
+      </c>
+      <c r="F26" s="26">
+        <f>COUNTIF(Tests!$G$5:$G$46,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G26" s="26">
+        <f>COUNTIF(Tests!$G$5:$G$46,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H26" s="26" t="n"/>
+    </row>
+    <row r="27"/>
+    <row r="28">
+      <c r="A28" s="27" t="inlineStr">
         <is>
           <t>Un test peut couvrir plusieurs PR : il compte pour chacune. « Validée » = tous les tests de la PR en OK ou Non testable. Un test « Partiel » corrigé depuis reste « En cours » jusqu'à ce que tu le refasses.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H4:H24">
+  <conditionalFormatting sqref="H4:H25">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="1">
       <formula>"Validée"</formula>
     </cfRule>
@@ -3594,7 +3742,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="16.5" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Recette : lien du build du 31/10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MoqekrFvgrWkuAe5NHnE5A
</commit_message>
<xml_diff>
--- a/docs/recette/RECETTE_PR_17-37.xlsx
+++ b/docs/recette/RECETTE_PR_17-37.xlsx
@@ -3603,7 +3603,6 @@
       </c>
       <c r="H26" s="26" t="n"/>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
@@ -3726,7 +3725,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>https://github.com/Herve-obe/VERIFLOW-v4/actions/runs/40517638115 (artefact veriflow-windows-latest, build du 27/10).</t>
+          <t>https://github.com/Herve-obe/VERIFLOW-v4/actions/runs/41209261957 (artefact veriflow-windows-latest, build du 31/10).</t>
         </is>
       </c>
     </row>
@@ -3742,6 +3741,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="16.5" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Recette : tests 43 à 50 (PR 41, avertissement batterie)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MoqekrFvgrWkuAe5NHnE5A
</commit_message>
<xml_diff>
--- a/docs/recette/RECETTE_PR_17-37.xlsx
+++ b/docs/recette/RECETTE_PR_17-37.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Légende" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tests'!$A$4:$J$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tests'!$A$4:$J$54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Tests'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -749,7 +749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:J54"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -766,7 +766,7 @@
     <row r="1" ht="18" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Recette VERIFLOW : PR 17 à 39 (build de la branche claude/recette, Windows 11)</t>
+          <t>Recette VERIFLOW : PR 17 à 41 (build de la branche claude/recette, Windows 11)</t>
         </is>
       </c>
     </row>
@@ -2696,8 +2696,312 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" s="29" t="n">
+        <v>43</v>
+      </c>
+      <c r="B47" s="30" t="inlineStr">
+        <is>
+          <t>C. OFFLOAD</t>
+        </is>
+      </c>
+      <c r="C47" s="29" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="D47" s="30" t="inlineStr">
+        <is>
+          <t>PC portable sur batterie (environ 50 %), grosse carte (copie de plus de 10 min) : préparer l'offload jusqu'aux contrôles avant copie.</t>
+        </is>
+      </c>
+      <c r="E47" s="30" t="inlineStr">
+        <is>
+          <t>Avertissement « Portable sur batterie (x %) et copie estimée à N min » dans les contrôles, puis à nouveau dans la confirmation de Lancer ; on peut continuer.</t>
+        </is>
+      </c>
+      <c r="F47" s="31" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="G47" s="31" t="n"/>
+      <c r="H47" s="32" t="n"/>
+      <c r="I47" s="33" t="n"/>
+      <c r="J47" s="34" t="inlineStr">
+        <is>
+          <t>Nouveau test (PR 41, 31/10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="29" t="n">
+        <v>44</v>
+      </c>
+      <c r="B48" s="30" t="inlineStr">
+        <is>
+          <t>C. OFFLOAD</t>
+        </is>
+      </c>
+      <c r="C48" s="29" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="D48" s="30" t="inlineStr">
+        <is>
+          <t>Même préparation, PC branché sur secteur.</t>
+        </is>
+      </c>
+      <c r="E48" s="30" t="inlineStr">
+        <is>
+          <t>Aucun avertissement batterie.</t>
+        </is>
+      </c>
+      <c r="F48" s="31" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="G48" s="31" t="n"/>
+      <c r="H48" s="32" t="n"/>
+      <c r="I48" s="33" t="n"/>
+      <c r="J48" s="34" t="inlineStr">
+        <is>
+          <t>Nouveau test (PR 41, 31/10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="29" t="n">
+        <v>45</v>
+      </c>
+      <c r="B49" s="30" t="inlineStr">
+        <is>
+          <t>C. OFFLOAD</t>
+        </is>
+      </c>
+      <c r="C49" s="29" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="D49" s="30" t="inlineStr">
+        <is>
+          <t>Préparer l'offload sur secteur, débrancher le chargeur, puis cliquer sur Lancer.</t>
+        </is>
+      </c>
+      <c r="E49" s="30" t="inlineStr">
+        <is>
+          <t>La confirmation affiche l'avertissement batterie (réévalué au clic).</t>
+        </is>
+      </c>
+      <c r="F49" s="31" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="G49" s="31" t="n"/>
+      <c r="H49" s="32" t="n"/>
+      <c r="I49" s="33" t="n"/>
+      <c r="J49" s="34" t="inlineStr">
+        <is>
+          <t>Nouveau test (PR 41, 31/10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="29" t="n">
+        <v>46</v>
+      </c>
+      <c r="B50" s="30" t="inlineStr">
+        <is>
+          <t>C. OFFLOAD</t>
+        </is>
+      </c>
+      <c r="C50" s="29" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="D50" s="30" t="inlineStr">
+        <is>
+          <t>Lancer une copie longue sur secteur, puis débrancher le chargeur pendant la copie.</t>
+        </is>
+      </c>
+      <c r="E50" s="30" t="inlineStr">
+        <is>
+          <t>Bandeau « passé sur batterie pendant la copie » en moins d'une minute ; bouton Fermer ; le bandeau disparaît si on rebranche.</t>
+        </is>
+      </c>
+      <c r="F50" s="31" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="G50" s="31" t="n"/>
+      <c r="H50" s="32" t="n"/>
+      <c r="I50" s="33" t="n"/>
+      <c r="J50" s="34" t="inlineStr">
+        <is>
+          <t>Nouveau test (PR 41, 31/10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="29" t="n">
+        <v>47</v>
+      </c>
+      <c r="B51" s="30" t="inlineStr">
+        <is>
+          <t>C. OFFLOAD</t>
+        </is>
+      </c>
+      <c r="C51" s="29" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="D51" s="30" t="inlineStr">
+        <is>
+          <t>Lancer une copie longue directement sur batterie.</t>
+        </is>
+      </c>
+      <c r="E51" s="30" t="inlineStr">
+        <is>
+          <t>Bandeau « Copie en cours sur batterie, fin estimée dans N min » au plus tard une minute après le début, une seule fois.</t>
+        </is>
+      </c>
+      <c r="F51" s="31" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="G51" s="31" t="n"/>
+      <c r="H51" s="32" t="n"/>
+      <c r="I51" s="33" t="n"/>
+      <c r="J51" s="34" t="inlineStr">
+        <is>
+          <t>Nouveau test (PR 41, 31/10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="29" t="n">
+        <v>48</v>
+      </c>
+      <c r="B52" s="30" t="inlineStr">
+        <is>
+          <t>C. OFFLOAD</t>
+        </is>
+      </c>
+      <c r="C52" s="29" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="D52" s="30" t="inlineStr">
+        <is>
+          <t>Batterie sous 20 %, petite carte (copie courte).</t>
+        </is>
+      </c>
+      <c r="E52" s="30" t="inlineStr">
+        <is>
+          <t>Avertissement « Batterie faible (x %) » avant la copie.</t>
+        </is>
+      </c>
+      <c r="F52" s="31" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="G52" s="31" t="n"/>
+      <c r="H52" s="32" t="n"/>
+      <c r="I52" s="33" t="n"/>
+      <c r="J52" s="34" t="inlineStr">
+        <is>
+          <t>Nouveau test (PR 41, 31/10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="29" t="n">
+        <v>49</v>
+      </c>
+      <c r="B53" s="30" t="inlineStr">
+        <is>
+          <t>C. OFFLOAD</t>
+        </is>
+      </c>
+      <c r="C53" s="29" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="D53" s="30" t="inlineStr">
+        <is>
+          <t>PC fixe (ou portable sans batterie) : préparer un offload.</t>
+        </is>
+      </c>
+      <c r="E53" s="30" t="inlineStr">
+        <is>
+          <t>Aucun avertissement ; contrôles avant copie aussi rapides qu'avant.</t>
+        </is>
+      </c>
+      <c r="F53" s="31" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="G53" s="31" t="n"/>
+      <c r="H53" s="32" t="n"/>
+      <c r="I53" s="33" t="n"/>
+      <c r="J53" s="34" t="inlineStr">
+        <is>
+          <t>Nouveau test (PR 41, 31/10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="29" t="n">
+        <v>50</v>
+      </c>
+      <c r="B54" s="30" t="inlineStr">
+        <is>
+          <t>C. OFFLOAD</t>
+        </is>
+      </c>
+      <c r="C54" s="29" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="D54" s="30" t="inlineStr">
+        <is>
+          <t>Interface en anglais : refaire le test 43.</t>
+        </is>
+      </c>
+      <c r="E54" s="30" t="inlineStr">
+        <is>
+          <t>Texte anglais lisible, pourcentage écrit « 50% », aucun {percent} ni {minutes} visible.</t>
+        </is>
+      </c>
+      <c r="F54" s="31" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="G54" s="31" t="n"/>
+      <c r="H54" s="32" t="n"/>
+      <c r="I54" s="33" t="n"/>
+      <c r="J54" s="34" t="inlineStr">
+        <is>
+          <t>Nouveau test (PR 41, 31/10).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:J46">
+  <autoFilter ref="A4:J54">
     <filterColumn colId="6" hiddenButton="0" showButton="1">
       <filters blank="1">
         <filter val="KO"/>
@@ -2705,7 +3009,7 @@
       </filters>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="G5:G46">
+  <conditionalFormatting sqref="G5:G54">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="6">
       <formula>"OK"</formula>
     </cfRule>
@@ -2720,13 +3024,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="F5:F46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F5:F54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Oui,Non"</formula1>
     </dataValidation>
-    <dataValidation sqref="G5:G46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,KO,Partiel,Non testable"</formula1>
     </dataValidation>
-    <dataValidation sqref="H5:H46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date" operator="greaterThan">
+    <dataValidation sqref="H5:H54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date" operator="greaterThan">
       <formula1>DATE(2026,1,1)</formula1>
     </dataValidation>
   </dataValidations>
@@ -2741,7 +3045,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2808,27 +3112,27 @@
         </is>
       </c>
       <c r="B4" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A4&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$54,"*"&amp;A4&amp;"*")</f>
         <v/>
       </c>
       <c r="C4" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A4&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A4&amp;"*",Tests!$F$5:$F$54,"Oui")</f>
         <v/>
       </c>
       <c r="D4" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A4&amp;"*",Tests!$G$5:$G$46,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A4&amp;"*",Tests!$G$5:$G$54,"OK")</f>
         <v/>
       </c>
       <c r="E4" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A4&amp;"*",Tests!$G$5:$G$46,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A4&amp;"*",Tests!$G$5:$G$54,"KO")</f>
         <v/>
       </c>
       <c r="F4" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A4&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A4&amp;"*",Tests!$G$5:$G$54,"Partiel")</f>
         <v/>
       </c>
       <c r="G4" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A4&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A4&amp;"*",Tests!$G$5:$G$54,"Non testable")</f>
         <v/>
       </c>
       <c r="H4" s="25">
@@ -2843,27 +3147,27 @@
         </is>
       </c>
       <c r="B5" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A5&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$54,"*"&amp;A5&amp;"*")</f>
         <v/>
       </c>
       <c r="C5" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A5&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A5&amp;"*",Tests!$F$5:$F$54,"Oui")</f>
         <v/>
       </c>
       <c r="D5" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A5&amp;"*",Tests!$G$5:$G$46,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A5&amp;"*",Tests!$G$5:$G$54,"OK")</f>
         <v/>
       </c>
       <c r="E5" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A5&amp;"*",Tests!$G$5:$G$46,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A5&amp;"*",Tests!$G$5:$G$54,"KO")</f>
         <v/>
       </c>
       <c r="F5" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A5&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A5&amp;"*",Tests!$G$5:$G$54,"Partiel")</f>
         <v/>
       </c>
       <c r="G5" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A5&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A5&amp;"*",Tests!$G$5:$G$54,"Non testable")</f>
         <v/>
       </c>
       <c r="H5" s="25">
@@ -2878,27 +3182,27 @@
         </is>
       </c>
       <c r="B6" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A6&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$54,"*"&amp;A6&amp;"*")</f>
         <v/>
       </c>
       <c r="C6" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A6&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A6&amp;"*",Tests!$F$5:$F$54,"Oui")</f>
         <v/>
       </c>
       <c r="D6" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A6&amp;"*",Tests!$G$5:$G$46,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A6&amp;"*",Tests!$G$5:$G$54,"OK")</f>
         <v/>
       </c>
       <c r="E6" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A6&amp;"*",Tests!$G$5:$G$46,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A6&amp;"*",Tests!$G$5:$G$54,"KO")</f>
         <v/>
       </c>
       <c r="F6" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A6&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A6&amp;"*",Tests!$G$5:$G$54,"Partiel")</f>
         <v/>
       </c>
       <c r="G6" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A6&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A6&amp;"*",Tests!$G$5:$G$54,"Non testable")</f>
         <v/>
       </c>
       <c r="H6" s="25">
@@ -2913,27 +3217,27 @@
         </is>
       </c>
       <c r="B7" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A7&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$54,"*"&amp;A7&amp;"*")</f>
         <v/>
       </c>
       <c r="C7" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A7&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A7&amp;"*",Tests!$F$5:$F$54,"Oui")</f>
         <v/>
       </c>
       <c r="D7" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A7&amp;"*",Tests!$G$5:$G$46,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A7&amp;"*",Tests!$G$5:$G$54,"OK")</f>
         <v/>
       </c>
       <c r="E7" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A7&amp;"*",Tests!$G$5:$G$46,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A7&amp;"*",Tests!$G$5:$G$54,"KO")</f>
         <v/>
       </c>
       <c r="F7" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A7&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A7&amp;"*",Tests!$G$5:$G$54,"Partiel")</f>
         <v/>
       </c>
       <c r="G7" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A7&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A7&amp;"*",Tests!$G$5:$G$54,"Non testable")</f>
         <v/>
       </c>
       <c r="H7" s="25">
@@ -2948,27 +3252,27 @@
         </is>
       </c>
       <c r="B8" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A8&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$54,"*"&amp;A8&amp;"*")</f>
         <v/>
       </c>
       <c r="C8" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A8&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A8&amp;"*",Tests!$F$5:$F$54,"Oui")</f>
         <v/>
       </c>
       <c r="D8" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A8&amp;"*",Tests!$G$5:$G$46,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A8&amp;"*",Tests!$G$5:$G$54,"OK")</f>
         <v/>
       </c>
       <c r="E8" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A8&amp;"*",Tests!$G$5:$G$46,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A8&amp;"*",Tests!$G$5:$G$54,"KO")</f>
         <v/>
       </c>
       <c r="F8" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A8&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A8&amp;"*",Tests!$G$5:$G$54,"Partiel")</f>
         <v/>
       </c>
       <c r="G8" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A8&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A8&amp;"*",Tests!$G$5:$G$54,"Non testable")</f>
         <v/>
       </c>
       <c r="H8" s="25">
@@ -2983,27 +3287,27 @@
         </is>
       </c>
       <c r="B9" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A9&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$54,"*"&amp;A9&amp;"*")</f>
         <v/>
       </c>
       <c r="C9" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A9&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A9&amp;"*",Tests!$F$5:$F$54,"Oui")</f>
         <v/>
       </c>
       <c r="D9" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A9&amp;"*",Tests!$G$5:$G$46,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A9&amp;"*",Tests!$G$5:$G$54,"OK")</f>
         <v/>
       </c>
       <c r="E9" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A9&amp;"*",Tests!$G$5:$G$46,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A9&amp;"*",Tests!$G$5:$G$54,"KO")</f>
         <v/>
       </c>
       <c r="F9" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A9&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A9&amp;"*",Tests!$G$5:$G$54,"Partiel")</f>
         <v/>
       </c>
       <c r="G9" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A9&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A9&amp;"*",Tests!$G$5:$G$54,"Non testable")</f>
         <v/>
       </c>
       <c r="H9" s="25">
@@ -3018,27 +3322,27 @@
         </is>
       </c>
       <c r="B10" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A10&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$54,"*"&amp;A10&amp;"*")</f>
         <v/>
       </c>
       <c r="C10" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A10&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A10&amp;"*",Tests!$F$5:$F$54,"Oui")</f>
         <v/>
       </c>
       <c r="D10" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A10&amp;"*",Tests!$G$5:$G$46,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A10&amp;"*",Tests!$G$5:$G$54,"OK")</f>
         <v/>
       </c>
       <c r="E10" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A10&amp;"*",Tests!$G$5:$G$46,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A10&amp;"*",Tests!$G$5:$G$54,"KO")</f>
         <v/>
       </c>
       <c r="F10" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A10&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A10&amp;"*",Tests!$G$5:$G$54,"Partiel")</f>
         <v/>
       </c>
       <c r="G10" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A10&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A10&amp;"*",Tests!$G$5:$G$54,"Non testable")</f>
         <v/>
       </c>
       <c r="H10" s="25">
@@ -3053,27 +3357,27 @@
         </is>
       </c>
       <c r="B11" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A11&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$54,"*"&amp;A11&amp;"*")</f>
         <v/>
       </c>
       <c r="C11" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A11&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A11&amp;"*",Tests!$F$5:$F$54,"Oui")</f>
         <v/>
       </c>
       <c r="D11" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A11&amp;"*",Tests!$G$5:$G$46,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A11&amp;"*",Tests!$G$5:$G$54,"OK")</f>
         <v/>
       </c>
       <c r="E11" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A11&amp;"*",Tests!$G$5:$G$46,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A11&amp;"*",Tests!$G$5:$G$54,"KO")</f>
         <v/>
       </c>
       <c r="F11" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A11&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A11&amp;"*",Tests!$G$5:$G$54,"Partiel")</f>
         <v/>
       </c>
       <c r="G11" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A11&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A11&amp;"*",Tests!$G$5:$G$54,"Non testable")</f>
         <v/>
       </c>
       <c r="H11" s="25">
@@ -3088,27 +3392,27 @@
         </is>
       </c>
       <c r="B12" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A12&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$54,"*"&amp;A12&amp;"*")</f>
         <v/>
       </c>
       <c r="C12" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A12&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A12&amp;"*",Tests!$F$5:$F$54,"Oui")</f>
         <v/>
       </c>
       <c r="D12" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A12&amp;"*",Tests!$G$5:$G$46,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A12&amp;"*",Tests!$G$5:$G$54,"OK")</f>
         <v/>
       </c>
       <c r="E12" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A12&amp;"*",Tests!$G$5:$G$46,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A12&amp;"*",Tests!$G$5:$G$54,"KO")</f>
         <v/>
       </c>
       <c r="F12" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A12&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A12&amp;"*",Tests!$G$5:$G$54,"Partiel")</f>
         <v/>
       </c>
       <c r="G12" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A12&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A12&amp;"*",Tests!$G$5:$G$54,"Non testable")</f>
         <v/>
       </c>
       <c r="H12" s="25">
@@ -3123,27 +3427,27 @@
         </is>
       </c>
       <c r="B13" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A13&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$54,"*"&amp;A13&amp;"*")</f>
         <v/>
       </c>
       <c r="C13" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A13&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A13&amp;"*",Tests!$F$5:$F$54,"Oui")</f>
         <v/>
       </c>
       <c r="D13" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A13&amp;"*",Tests!$G$5:$G$46,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A13&amp;"*",Tests!$G$5:$G$54,"OK")</f>
         <v/>
       </c>
       <c r="E13" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A13&amp;"*",Tests!$G$5:$G$46,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A13&amp;"*",Tests!$G$5:$G$54,"KO")</f>
         <v/>
       </c>
       <c r="F13" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A13&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A13&amp;"*",Tests!$G$5:$G$54,"Partiel")</f>
         <v/>
       </c>
       <c r="G13" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A13&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A13&amp;"*",Tests!$G$5:$G$54,"Non testable")</f>
         <v/>
       </c>
       <c r="H13" s="25">
@@ -3158,27 +3462,27 @@
         </is>
       </c>
       <c r="B14" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A14&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$54,"*"&amp;A14&amp;"*")</f>
         <v/>
       </c>
       <c r="C14" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A14&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A14&amp;"*",Tests!$F$5:$F$54,"Oui")</f>
         <v/>
       </c>
       <c r="D14" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A14&amp;"*",Tests!$G$5:$G$46,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A14&amp;"*",Tests!$G$5:$G$54,"OK")</f>
         <v/>
       </c>
       <c r="E14" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A14&amp;"*",Tests!$G$5:$G$46,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A14&amp;"*",Tests!$G$5:$G$54,"KO")</f>
         <v/>
       </c>
       <c r="F14" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A14&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A14&amp;"*",Tests!$G$5:$G$54,"Partiel")</f>
         <v/>
       </c>
       <c r="G14" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A14&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A14&amp;"*",Tests!$G$5:$G$54,"Non testable")</f>
         <v/>
       </c>
       <c r="H14" s="25">
@@ -3193,27 +3497,27 @@
         </is>
       </c>
       <c r="B15" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A15&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$54,"*"&amp;A15&amp;"*")</f>
         <v/>
       </c>
       <c r="C15" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A15&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A15&amp;"*",Tests!$F$5:$F$54,"Oui")</f>
         <v/>
       </c>
       <c r="D15" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A15&amp;"*",Tests!$G$5:$G$46,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A15&amp;"*",Tests!$G$5:$G$54,"OK")</f>
         <v/>
       </c>
       <c r="E15" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A15&amp;"*",Tests!$G$5:$G$46,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A15&amp;"*",Tests!$G$5:$G$54,"KO")</f>
         <v/>
       </c>
       <c r="F15" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A15&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A15&amp;"*",Tests!$G$5:$G$54,"Partiel")</f>
         <v/>
       </c>
       <c r="G15" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A15&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A15&amp;"*",Tests!$G$5:$G$54,"Non testable")</f>
         <v/>
       </c>
       <c r="H15" s="25">
@@ -3228,27 +3532,27 @@
         </is>
       </c>
       <c r="B16" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A16&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$54,"*"&amp;A16&amp;"*")</f>
         <v/>
       </c>
       <c r="C16" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A16&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A16&amp;"*",Tests!$F$5:$F$54,"Oui")</f>
         <v/>
       </c>
       <c r="D16" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A16&amp;"*",Tests!$G$5:$G$46,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A16&amp;"*",Tests!$G$5:$G$54,"OK")</f>
         <v/>
       </c>
       <c r="E16" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A16&amp;"*",Tests!$G$5:$G$46,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A16&amp;"*",Tests!$G$5:$G$54,"KO")</f>
         <v/>
       </c>
       <c r="F16" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A16&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A16&amp;"*",Tests!$G$5:$G$54,"Partiel")</f>
         <v/>
       </c>
       <c r="G16" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A16&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A16&amp;"*",Tests!$G$5:$G$54,"Non testable")</f>
         <v/>
       </c>
       <c r="H16" s="25">
@@ -3263,27 +3567,27 @@
         </is>
       </c>
       <c r="B17" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A17&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$54,"*"&amp;A17&amp;"*")</f>
         <v/>
       </c>
       <c r="C17" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A17&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A17&amp;"*",Tests!$F$5:$F$54,"Oui")</f>
         <v/>
       </c>
       <c r="D17" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A17&amp;"*",Tests!$G$5:$G$46,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A17&amp;"*",Tests!$G$5:$G$54,"OK")</f>
         <v/>
       </c>
       <c r="E17" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A17&amp;"*",Tests!$G$5:$G$46,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A17&amp;"*",Tests!$G$5:$G$54,"KO")</f>
         <v/>
       </c>
       <c r="F17" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A17&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A17&amp;"*",Tests!$G$5:$G$54,"Partiel")</f>
         <v/>
       </c>
       <c r="G17" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A17&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A17&amp;"*",Tests!$G$5:$G$54,"Non testable")</f>
         <v/>
       </c>
       <c r="H17" s="25">
@@ -3298,27 +3602,27 @@
         </is>
       </c>
       <c r="B18" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A18&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$54,"*"&amp;A18&amp;"*")</f>
         <v/>
       </c>
       <c r="C18" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A18&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A18&amp;"*",Tests!$F$5:$F$54,"Oui")</f>
         <v/>
       </c>
       <c r="D18" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A18&amp;"*",Tests!$G$5:$G$46,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A18&amp;"*",Tests!$G$5:$G$54,"OK")</f>
         <v/>
       </c>
       <c r="E18" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A18&amp;"*",Tests!$G$5:$G$46,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A18&amp;"*",Tests!$G$5:$G$54,"KO")</f>
         <v/>
       </c>
       <c r="F18" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A18&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A18&amp;"*",Tests!$G$5:$G$54,"Partiel")</f>
         <v/>
       </c>
       <c r="G18" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A18&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A18&amp;"*",Tests!$G$5:$G$54,"Non testable")</f>
         <v/>
       </c>
       <c r="H18" s="25">
@@ -3333,27 +3637,27 @@
         </is>
       </c>
       <c r="B19" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A19&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$54,"*"&amp;A19&amp;"*")</f>
         <v/>
       </c>
       <c r="C19" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A19&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A19&amp;"*",Tests!$F$5:$F$54,"Oui")</f>
         <v/>
       </c>
       <c r="D19" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A19&amp;"*",Tests!$G$5:$G$46,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A19&amp;"*",Tests!$G$5:$G$54,"OK")</f>
         <v/>
       </c>
       <c r="E19" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A19&amp;"*",Tests!$G$5:$G$46,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A19&amp;"*",Tests!$G$5:$G$54,"KO")</f>
         <v/>
       </c>
       <c r="F19" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A19&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A19&amp;"*",Tests!$G$5:$G$54,"Partiel")</f>
         <v/>
       </c>
       <c r="G19" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A19&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A19&amp;"*",Tests!$G$5:$G$54,"Non testable")</f>
         <v/>
       </c>
       <c r="H19" s="25">
@@ -3368,27 +3672,27 @@
         </is>
       </c>
       <c r="B20" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A20&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$54,"*"&amp;A20&amp;"*")</f>
         <v/>
       </c>
       <c r="C20" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A20&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A20&amp;"*",Tests!$F$5:$F$54,"Oui")</f>
         <v/>
       </c>
       <c r="D20" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A20&amp;"*",Tests!$G$5:$G$46,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A20&amp;"*",Tests!$G$5:$G$54,"OK")</f>
         <v/>
       </c>
       <c r="E20" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A20&amp;"*",Tests!$G$5:$G$46,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A20&amp;"*",Tests!$G$5:$G$54,"KO")</f>
         <v/>
       </c>
       <c r="F20" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A20&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A20&amp;"*",Tests!$G$5:$G$54,"Partiel")</f>
         <v/>
       </c>
       <c r="G20" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A20&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A20&amp;"*",Tests!$G$5:$G$54,"Non testable")</f>
         <v/>
       </c>
       <c r="H20" s="25">
@@ -3403,27 +3707,27 @@
         </is>
       </c>
       <c r="B21" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A21&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$54,"*"&amp;A21&amp;"*")</f>
         <v/>
       </c>
       <c r="C21" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A21&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A21&amp;"*",Tests!$F$5:$F$54,"Oui")</f>
         <v/>
       </c>
       <c r="D21" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A21&amp;"*",Tests!$G$5:$G$46,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A21&amp;"*",Tests!$G$5:$G$54,"OK")</f>
         <v/>
       </c>
       <c r="E21" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A21&amp;"*",Tests!$G$5:$G$46,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A21&amp;"*",Tests!$G$5:$G$54,"KO")</f>
         <v/>
       </c>
       <c r="F21" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A21&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A21&amp;"*",Tests!$G$5:$G$54,"Partiel")</f>
         <v/>
       </c>
       <c r="G21" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A21&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A21&amp;"*",Tests!$G$5:$G$54,"Non testable")</f>
         <v/>
       </c>
       <c r="H21" s="25">
@@ -3438,27 +3742,27 @@
         </is>
       </c>
       <c r="B22" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A22&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$54,"*"&amp;A22&amp;"*")</f>
         <v/>
       </c>
       <c r="C22" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A22&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A22&amp;"*",Tests!$F$5:$F$54,"Oui")</f>
         <v/>
       </c>
       <c r="D22" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A22&amp;"*",Tests!$G$5:$G$46,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A22&amp;"*",Tests!$G$5:$G$54,"OK")</f>
         <v/>
       </c>
       <c r="E22" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A22&amp;"*",Tests!$G$5:$G$46,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A22&amp;"*",Tests!$G$5:$G$54,"KO")</f>
         <v/>
       </c>
       <c r="F22" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A22&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A22&amp;"*",Tests!$G$5:$G$54,"Partiel")</f>
         <v/>
       </c>
       <c r="G22" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A22&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A22&amp;"*",Tests!$G$5:$G$54,"Non testable")</f>
         <v/>
       </c>
       <c r="H22" s="25">
@@ -3473,27 +3777,27 @@
         </is>
       </c>
       <c r="B23" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$46,"*"&amp;A23&amp;"*")</f>
+        <f>COUNTIF(Tests!$C$5:$C$54,"*"&amp;A23&amp;"*")</f>
         <v/>
       </c>
       <c r="C23" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A23&amp;"*",Tests!$F$5:$F$46,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A23&amp;"*",Tests!$F$5:$F$54,"Oui")</f>
         <v/>
       </c>
       <c r="D23" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A23&amp;"*",Tests!$G$5:$G$46,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A23&amp;"*",Tests!$G$5:$G$54,"OK")</f>
         <v/>
       </c>
       <c r="E23" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A23&amp;"*",Tests!$G$5:$G$46,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A23&amp;"*",Tests!$G$5:$G$54,"KO")</f>
         <v/>
       </c>
       <c r="F23" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A23&amp;"*",Tests!$G$5:$G$46,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A23&amp;"*",Tests!$G$5:$G$54,"Partiel")</f>
         <v/>
       </c>
       <c r="G23" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,"*"&amp;A23&amp;"*",Tests!$G$5:$G$46,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A23&amp;"*",Tests!$G$5:$G$54,"Non testable")</f>
         <v/>
       </c>
       <c r="H23" s="25">
@@ -3504,31 +3808,31 @@
     <row r="24">
       <c r="A24" s="25" t="inlineStr">
         <is>
-          <t>5 (en attente)</t>
+          <t>41</t>
         </is>
       </c>
       <c r="B24" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$46,A24)</f>
+        <f>COUNTIF(Tests!$C$5:$C$54,"*"&amp;A24&amp;"*")</f>
         <v/>
       </c>
       <c r="C24" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,A24,Tests!$F$5:$F$46,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A24&amp;"*",Tests!$F$5:$F$54,"Oui")</f>
         <v/>
       </c>
       <c r="D24" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,A24,Tests!$G$5:$G$46,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A24&amp;"*",Tests!$G$5:$G$54,"OK")</f>
         <v/>
       </c>
       <c r="E24" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,A24,Tests!$G$5:$G$46,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A24&amp;"*",Tests!$G$5:$G$54,"KO")</f>
         <v/>
       </c>
       <c r="F24" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,A24,Tests!$G$5:$G$46,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A24&amp;"*",Tests!$G$5:$G$54,"Partiel")</f>
         <v/>
       </c>
       <c r="G24" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,A24,Tests!$G$5:$G$46,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,"*"&amp;A24&amp;"*",Tests!$G$5:$G$54,"Non testable")</f>
         <v/>
       </c>
       <c r="H24" s="25">
@@ -3539,31 +3843,31 @@
     <row r="25">
       <c r="A25" s="25" t="inlineStr">
         <is>
-          <t>SYNC</t>
+          <t>5 (en attente)</t>
         </is>
       </c>
       <c r="B25" s="25">
-        <f>COUNTIF(Tests!$C$5:$C$46,A25)</f>
+        <f>COUNTIF(Tests!$C$5:$C$54,A25)</f>
         <v/>
       </c>
       <c r="C25" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,A25,Tests!$F$5:$F$46,"Oui")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,A25,Tests!$F$5:$F$54,"Oui")</f>
         <v/>
       </c>
       <c r="D25" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,A25,Tests!$G$5:$G$46,"OK")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,A25,Tests!$G$5:$G$54,"OK")</f>
         <v/>
       </c>
       <c r="E25" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,A25,Tests!$G$5:$G$46,"KO")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,A25,Tests!$G$5:$G$54,"KO")</f>
         <v/>
       </c>
       <c r="F25" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,A25,Tests!$G$5:$G$46,"Partiel")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,A25,Tests!$G$5:$G$54,"Partiel")</f>
         <v/>
       </c>
       <c r="G25" s="25">
-        <f>COUNTIFS(Tests!$C$5:$C$46,A25,Tests!$G$5:$G$46,"Non testable")</f>
+        <f>COUNTIFS(Tests!$C$5:$C$54,A25,Tests!$G$5:$G$54,"Non testable")</f>
         <v/>
       </c>
       <c r="H25" s="25">
@@ -3572,46 +3876,82 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="26" t="inlineStr">
+      <c r="A26" s="25" t="inlineStr">
+        <is>
+          <t>SYNC</t>
+        </is>
+      </c>
+      <c r="B26" s="25">
+        <f>COUNTIF(Tests!$C$5:$C$54,A26)</f>
+        <v/>
+      </c>
+      <c r="C26" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$54,A26,Tests!$F$5:$F$54,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D26" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$54,A26,Tests!$G$5:$G$54,"OK")</f>
+        <v/>
+      </c>
+      <c r="E26" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$54,A26,Tests!$G$5:$G$54,"KO")</f>
+        <v/>
+      </c>
+      <c r="F26" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$54,A26,Tests!$G$5:$G$54,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G26" s="25">
+        <f>COUNTIFS(Tests!$C$5:$C$54,A26,Tests!$G$5:$G$54,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H26" s="25">
+        <f>IF(E26&gt;0,"À corriger",IF(D26+G26=B26,"Validée",IF(C26=0,"À tester","En cours")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="26" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B26" s="26">
-        <f>COUNTA(Tests!$A$5:$A$46)</f>
-        <v/>
-      </c>
-      <c r="C26" s="26">
-        <f>COUNTIF(Tests!$F$5:$F$46,"Oui")</f>
-        <v/>
-      </c>
-      <c r="D26" s="26">
-        <f>COUNTIF(Tests!$G$5:$G$46,"OK")</f>
-        <v/>
-      </c>
-      <c r="E26" s="26">
-        <f>COUNTIF(Tests!$G$5:$G$46,"KO")</f>
-        <v/>
-      </c>
-      <c r="F26" s="26">
-        <f>COUNTIF(Tests!$G$5:$G$46,"Partiel")</f>
-        <v/>
-      </c>
-      <c r="G26" s="26">
-        <f>COUNTIF(Tests!$G$5:$G$46,"Non testable")</f>
-        <v/>
-      </c>
-      <c r="H26" s="26" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="27" t="inlineStr">
+      <c r="B27" s="26">
+        <f>COUNTA(Tests!$A$5:$A$54)</f>
+        <v/>
+      </c>
+      <c r="C27" s="26">
+        <f>COUNTIF(Tests!$F$5:$F$54,"Oui")</f>
+        <v/>
+      </c>
+      <c r="D27" s="26">
+        <f>COUNTIF(Tests!$G$5:$G$54,"OK")</f>
+        <v/>
+      </c>
+      <c r="E27" s="26">
+        <f>COUNTIF(Tests!$G$5:$G$54,"KO")</f>
+        <v/>
+      </c>
+      <c r="F27" s="26">
+        <f>COUNTIF(Tests!$G$5:$G$54,"Partiel")</f>
+        <v/>
+      </c>
+      <c r="G27" s="26">
+        <f>COUNTIF(Tests!$G$5:$G$54,"Non testable")</f>
+        <v/>
+      </c>
+      <c r="H27" s="26" t="n"/>
+    </row>
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" s="27" t="inlineStr">
         <is>
           <t>Un test peut couvrir plusieurs PR : il compte pour chacune. « Validée » = tous les tests de la PR en OK ou Non testable. Un test « Partiel » corrigé depuis reste « En cours » jusqu'à ce que tu le refasses.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H4:H25">
+  <conditionalFormatting sqref="H4:H26">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="1">
       <formula>"Validée"</formula>
     </cfRule>
@@ -3741,7 +4081,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="16.5" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Recette : lien du build avec la PR 41
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MoqekrFvgrWkuAe5NHnE5A
</commit_message>
<xml_diff>
--- a/docs/recette/RECETTE_PR_17-37.xlsx
+++ b/docs/recette/RECETTE_PR_17-37.xlsx
@@ -3942,7 +3942,6 @@
       </c>
       <c r="H27" s="26" t="n"/>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
         <is>
@@ -4065,7 +4064,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>https://github.com/Herve-obe/VERIFLOW-v4/actions/runs/41209261957 (artefact veriflow-windows-latest, build du 31/10).</t>
+          <t>https://github.com/Herve-obe/VERIFLOW-v4/actions/runs/41215916672 (artefact veriflow-windows-latest, build du 31/10 avec PR 39 et 41).</t>
         </is>
       </c>
     </row>
@@ -4081,6 +4080,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="16.5" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
         <is>

</xml_diff>